<commit_message>
Atualiza├º├úo autom├ítica 2025-10-14 11:06
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="329" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D82B8A67-AE72-4A2A-AE15-832CB1E81081}"/>
+  <xr:revisionPtr revIDLastSave="641" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5571D5BF-7362-4C43-BC82-CBB6A8D3CA90}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7943" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8066" uniqueCount="335">
   <si>
     <t>Data</t>
   </si>
@@ -1039,6 +1039,12 @@
   <si>
     <t>EDENEY</t>
   </si>
+  <si>
+    <t>POSTO ITAJAO</t>
+  </si>
+  <si>
+    <t>POSTO SOARES</t>
+  </si>
 </sst>
 </file>
 
@@ -1179,7 +1185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1235,7 +1241,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1245,7 +1251,6 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -1597,7 +1602,18 @@
     <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" s="33" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+      <c r="H1"/>
+      <c r="I1"/>
+      <c r="J1"/>
+      <c r="K1"/>
+    </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
         <v>0</v>
@@ -70047,19 +70063,33 @@
       </c>
     </row>
     <row r="2131" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2131" s="18"/>
+      <c r="B2131" s="18">
+        <v>45938</v>
+      </c>
       <c r="C2131" s="1"/>
       <c r="D2131" s="1"/>
       <c r="E2131" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2131" s="1"/>
-      <c r="G2131" s="10"/>
-      <c r="H2131" s="3"/>
-      <c r="I2131" s="12"/>
-      <c r="J2131" s="7"/>
-      <c r="K2131" s="7"/>
+      <c r="F2131" s="1">
+        <v>46.94</v>
+      </c>
+      <c r="G2131" s="10">
+        <v>300</v>
+      </c>
+      <c r="H2131" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2131" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2131" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2131" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2132" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2132" s="18">
@@ -70352,124 +70382,236 @@
       </c>
     </row>
     <row r="2142" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2142" s="18"/>
+      <c r="B2142" s="18">
+        <v>45937</v>
+      </c>
       <c r="C2142" s="1"/>
       <c r="D2142" s="1"/>
       <c r="E2142" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2142" s="1"/>
-      <c r="G2142" s="10"/>
-      <c r="H2142" s="3"/>
-      <c r="I2142" s="12"/>
-      <c r="J2142" s="7"/>
-      <c r="K2142" s="7"/>
+      <c r="F2142" s="1">
+        <v>135.13999999999999</v>
+      </c>
+      <c r="G2142" s="10">
+        <v>850.03</v>
+      </c>
+      <c r="H2142" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2142" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2142" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2142" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2143" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2143" s="18"/>
+      <c r="B2143" s="18">
+        <v>45931</v>
+      </c>
       <c r="C2143" s="1"/>
       <c r="D2143" s="1"/>
       <c r="E2143" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2143" s="1"/>
-      <c r="G2143" s="10"/>
-      <c r="H2143" s="3"/>
-      <c r="I2143" s="12"/>
-      <c r="J2143" s="7"/>
-      <c r="K2143" s="7"/>
+      <c r="F2143" s="1">
+        <v>195.1</v>
+      </c>
+      <c r="G2143" s="10">
+        <v>1227.21</v>
+      </c>
+      <c r="H2143" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2143" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2143" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2143" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2144" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2144" s="18"/>
+      <c r="B2144" s="18">
+        <v>45931</v>
+      </c>
       <c r="C2144" s="1"/>
       <c r="D2144" s="1"/>
       <c r="E2144" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2144" s="1"/>
-      <c r="G2144" s="10"/>
-      <c r="H2144" s="3"/>
-      <c r="I2144" s="12"/>
-      <c r="J2144" s="7"/>
-      <c r="K2144" s="7"/>
+      <c r="F2144" s="1">
+        <v>50.084000000000003</v>
+      </c>
+      <c r="G2144" s="10">
+        <v>300</v>
+      </c>
+      <c r="H2144" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2144" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2144" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="K2144" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2145" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2145" s="18"/>
+      <c r="B2145" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2145" s="1"/>
       <c r="D2145" s="1"/>
       <c r="E2145" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2145" s="1"/>
-      <c r="G2145" s="10"/>
-      <c r="H2145" s="3"/>
-      <c r="I2145" s="12"/>
-      <c r="J2145" s="7"/>
-      <c r="K2145" s="7"/>
+      <c r="F2145" s="1">
+        <v>78.239999999999995</v>
+      </c>
+      <c r="G2145" s="10">
+        <v>500</v>
+      </c>
+      <c r="H2145" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2145" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2145" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2145" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2146" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2146" s="18"/>
+      <c r="B2146" s="18">
+        <v>45938</v>
+      </c>
       <c r="C2146" s="1"/>
       <c r="D2146" s="1"/>
       <c r="E2146" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2146" s="1"/>
-      <c r="G2146" s="10"/>
-      <c r="H2146" s="3"/>
-      <c r="I2146" s="12"/>
-      <c r="J2146" s="7"/>
-      <c r="K2146" s="7"/>
+      <c r="F2146" s="1">
+        <v>144.86000000000001</v>
+      </c>
+      <c r="G2146" s="10">
+        <v>911.21</v>
+      </c>
+      <c r="H2146" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2146" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2146" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2146" s="7" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="2147" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2147" s="18"/>
+      <c r="B2147" s="18">
+        <v>45941</v>
+      </c>
       <c r="C2147" s="1"/>
       <c r="D2147" s="1"/>
       <c r="E2147" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2147" s="1"/>
-      <c r="G2147" s="10"/>
-      <c r="H2147" s="3"/>
-      <c r="I2147" s="12"/>
-      <c r="J2147" s="7"/>
-      <c r="K2147" s="7"/>
+      <c r="F2147" s="1">
+        <v>99.17</v>
+      </c>
+      <c r="G2147" s="10">
+        <v>600</v>
+      </c>
+      <c r="H2147" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2147" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2147" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="K2147" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="2148" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2148" s="18"/>
+      <c r="B2148" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2148" s="1"/>
       <c r="D2148" s="1"/>
       <c r="E2148" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2148" s="1"/>
-      <c r="G2148" s="10"/>
-      <c r="H2148" s="3"/>
-      <c r="I2148" s="12"/>
-      <c r="J2148" s="7"/>
-      <c r="K2148" s="7"/>
+      <c r="F2148" s="1">
+        <v>153.18100000000001</v>
+      </c>
+      <c r="G2148" s="10">
+        <v>891.51</v>
+      </c>
+      <c r="H2148" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2148" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2148" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2148" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="2149" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2149" s="18"/>
+      <c r="B2149" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2149" s="1"/>
       <c r="D2149" s="1"/>
       <c r="E2149" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2149" s="1"/>
-      <c r="G2149" s="10"/>
-      <c r="H2149" s="3"/>
-      <c r="I2149" s="12"/>
-      <c r="J2149" s="7"/>
-      <c r="K2149" s="7"/>
+      <c r="F2149" s="1">
+        <v>147</v>
+      </c>
+      <c r="G2149" s="10">
+        <v>968.73</v>
+      </c>
+      <c r="H2149" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2149" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2149" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="K2149" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="2150" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2150" s="18">
@@ -70501,124 +70643,236 @@
       </c>
     </row>
     <row r="2151" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2151" s="18"/>
+      <c r="B2151" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2151" s="1"/>
       <c r="D2151" s="1"/>
       <c r="E2151" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2151" s="1"/>
-      <c r="G2151" s="10"/>
-      <c r="H2151" s="3"/>
-      <c r="I2151" s="12"/>
-      <c r="J2151" s="7"/>
-      <c r="K2151" s="7"/>
+      <c r="F2151" s="1">
+        <v>35.726999999999997</v>
+      </c>
+      <c r="G2151" s="10">
+        <v>207.93</v>
+      </c>
+      <c r="H2151" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2151" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2151" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2151" s="7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="2152" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2152" s="18"/>
+      <c r="B2152" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2152" s="1"/>
       <c r="D2152" s="1"/>
       <c r="E2152" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2152" s="1"/>
-      <c r="G2152" s="10"/>
-      <c r="H2152" s="3"/>
-      <c r="I2152" s="12"/>
-      <c r="J2152" s="7"/>
-      <c r="K2152" s="7"/>
+      <c r="F2152" s="1">
+        <v>160.53</v>
+      </c>
+      <c r="G2152" s="10">
+        <v>1021</v>
+      </c>
+      <c r="H2152" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2152" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2152" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="K2152" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2153" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2153" s="18"/>
+      <c r="B2153" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2153" s="1"/>
       <c r="D2153" s="1"/>
       <c r="E2153" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2153" s="1"/>
-      <c r="G2153" s="10"/>
-      <c r="H2153" s="3"/>
-      <c r="I2153" s="12"/>
-      <c r="J2153" s="7"/>
-      <c r="K2153" s="7"/>
+      <c r="F2153" s="1">
+        <v>165.83</v>
+      </c>
+      <c r="G2153" s="10">
+        <v>965.13</v>
+      </c>
+      <c r="H2153" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2153" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2153" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2153" s="7" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="2154" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2154" s="18"/>
+      <c r="B2154" s="18">
+        <v>45929</v>
+      </c>
       <c r="C2154" s="1"/>
       <c r="D2154" s="1"/>
       <c r="E2154" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2154" s="1"/>
-      <c r="G2154" s="10"/>
-      <c r="H2154" s="3"/>
-      <c r="I2154" s="12"/>
-      <c r="J2154" s="7"/>
-      <c r="K2154" s="7"/>
+      <c r="F2154" s="1">
+        <v>151.453</v>
+      </c>
+      <c r="G2154" s="10">
+        <v>881.45</v>
+      </c>
+      <c r="H2154" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2154" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2154" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2154" s="7" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="2155" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2155" s="18"/>
+      <c r="B2155" s="18">
+        <v>45938</v>
+      </c>
       <c r="C2155" s="1"/>
       <c r="D2155" s="1"/>
       <c r="E2155" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2155" s="1"/>
-      <c r="G2155" s="10"/>
-      <c r="H2155" s="3"/>
-      <c r="I2155" s="12"/>
-      <c r="J2155" s="7"/>
-      <c r="K2155" s="7"/>
+      <c r="F2155" s="1">
+        <v>154.06100000000001</v>
+      </c>
+      <c r="G2155" s="10">
+        <v>1015.26</v>
+      </c>
+      <c r="H2155" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2155" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2155" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="K2155" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="2156" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2156" s="18"/>
+      <c r="B2156" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2156" s="1"/>
       <c r="D2156" s="1"/>
       <c r="E2156" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2156" s="1"/>
-      <c r="G2156" s="10"/>
-      <c r="H2156" s="3"/>
-      <c r="I2156" s="12"/>
-      <c r="J2156" s="7"/>
-      <c r="K2156" s="7"/>
+      <c r="F2156" s="1">
+        <v>125.348</v>
+      </c>
+      <c r="G2156" s="10">
+        <v>729</v>
+      </c>
+      <c r="H2156" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2156" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2156" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2156" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="2157" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2157" s="18"/>
+      <c r="B2157" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2157" s="1"/>
       <c r="D2157" s="1"/>
       <c r="E2157" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2157" s="1"/>
-      <c r="G2157" s="10"/>
-      <c r="H2157" s="3"/>
-      <c r="I2157" s="12"/>
-      <c r="J2157" s="7"/>
-      <c r="K2157" s="7"/>
+      <c r="F2157" s="1">
+        <v>82.78</v>
+      </c>
+      <c r="G2157" s="10">
+        <v>500</v>
+      </c>
+      <c r="H2157" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2157" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2157" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="K2157" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2158" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2158" s="18"/>
+      <c r="B2158" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2158" s="1"/>
       <c r="D2158" s="1"/>
       <c r="E2158" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2158" s="1"/>
-      <c r="G2158" s="10"/>
-      <c r="H2158" s="3"/>
-      <c r="I2158" s="12"/>
-      <c r="J2158" s="7"/>
-      <c r="K2158" s="7"/>
+      <c r="F2158" s="1">
+        <v>117.745</v>
+      </c>
+      <c r="G2158" s="10">
+        <v>685.27</v>
+      </c>
+      <c r="H2158" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2158" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2158" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2158" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2159" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2159" s="18">
@@ -70650,19 +70904,33 @@
       </c>
     </row>
     <row r="2160" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2160" s="18"/>
+      <c r="B2160" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2160" s="1"/>
       <c r="D2160" s="1"/>
       <c r="E2160" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2160" s="1"/>
-      <c r="G2160" s="10"/>
-      <c r="H2160" s="3"/>
-      <c r="I2160" s="12"/>
-      <c r="J2160" s="7"/>
-      <c r="K2160" s="7"/>
+      <c r="F2160" s="1">
+        <v>162.72999999999999</v>
+      </c>
+      <c r="G2160" s="10">
+        <v>1046.4000000000001</v>
+      </c>
+      <c r="H2160" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2160" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2160" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2160" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2161" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2161" s="18">
@@ -70694,34 +70962,62 @@
       </c>
     </row>
     <row r="2162" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2162" s="18"/>
+      <c r="B2162" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2162" s="1"/>
       <c r="D2162" s="1"/>
       <c r="E2162" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2162" s="1"/>
-      <c r="G2162" s="10"/>
-      <c r="H2162" s="3"/>
-      <c r="I2162" s="12"/>
-      <c r="J2162" s="7"/>
-      <c r="K2162" s="7"/>
+      <c r="F2162" s="1">
+        <v>168.53800000000001</v>
+      </c>
+      <c r="G2162" s="10">
+        <v>980.89</v>
+      </c>
+      <c r="H2162" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2162" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2162" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2162" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2163" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2163" s="18"/>
+      <c r="B2163" s="18">
+        <v>45929</v>
+      </c>
       <c r="C2163" s="1"/>
       <c r="D2163" s="1"/>
       <c r="E2163" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2163" s="1"/>
-      <c r="G2163" s="10"/>
-      <c r="H2163" s="3"/>
-      <c r="I2163" s="12"/>
-      <c r="J2163" s="7"/>
-      <c r="K2163" s="7"/>
+      <c r="F2163" s="1">
+        <v>53.39</v>
+      </c>
+      <c r="G2163" s="10">
+        <v>325.14999999999998</v>
+      </c>
+      <c r="H2163" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2163" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2163" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2163" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2164" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2164" s="18">
@@ -70753,34 +71049,62 @@
       </c>
     </row>
     <row r="2165" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2165" s="18"/>
+      <c r="B2165" s="18">
+        <v>45936</v>
+      </c>
       <c r="C2165" s="1"/>
       <c r="D2165" s="1"/>
       <c r="E2165" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2165" s="1"/>
-      <c r="G2165" s="10"/>
-      <c r="H2165" s="3"/>
-      <c r="I2165" s="12"/>
-      <c r="J2165" s="7"/>
-      <c r="K2165" s="7"/>
+      <c r="F2165" s="1">
+        <v>82.58</v>
+      </c>
+      <c r="G2165" s="10">
+        <v>502.91</v>
+      </c>
+      <c r="H2165" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2165" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2165" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2165" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2166" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2166" s="18"/>
+      <c r="B2166" s="18">
+        <v>45924</v>
+      </c>
       <c r="C2166" s="1"/>
       <c r="D2166" s="1"/>
       <c r="E2166" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2166" s="1"/>
-      <c r="G2166" s="10"/>
-      <c r="H2166" s="3"/>
-      <c r="I2166" s="12"/>
-      <c r="J2166" s="7"/>
-      <c r="K2166" s="7"/>
+      <c r="F2166" s="1">
+        <v>137.321</v>
+      </c>
+      <c r="G2166" s="10">
+        <v>836.28</v>
+      </c>
+      <c r="H2166" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2166" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2166" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2166" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2167" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2167" s="18">
@@ -70838,49 +71162,91 @@
       </c>
     </row>
     <row r="2169" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2169" s="18"/>
+      <c r="B2169" s="18">
+        <v>45930</v>
+      </c>
       <c r="C2169" s="1"/>
       <c r="D2169" s="1"/>
       <c r="E2169" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2169" s="1"/>
-      <c r="G2169" s="10"/>
-      <c r="H2169" s="3"/>
-      <c r="I2169" s="12"/>
-      <c r="J2169" s="7"/>
-      <c r="K2169" s="7"/>
+      <c r="F2169" s="1">
+        <v>68</v>
+      </c>
+      <c r="G2169" s="10">
+        <v>719.96</v>
+      </c>
+      <c r="H2169" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2169" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2169" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2169" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2170" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2170" s="18"/>
+      <c r="B2170" s="18">
+        <v>45930</v>
+      </c>
       <c r="C2170" s="1"/>
       <c r="D2170" s="1"/>
       <c r="E2170" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2170" s="1"/>
-      <c r="G2170" s="10"/>
-      <c r="H2170" s="3"/>
-      <c r="I2170" s="12"/>
-      <c r="J2170" s="7"/>
-      <c r="K2170" s="7"/>
+      <c r="F2170" s="1">
+        <v>137.321</v>
+      </c>
+      <c r="G2170" s="10">
+        <v>836.28</v>
+      </c>
+      <c r="H2170" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2170" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2170" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2170" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2171" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2171" s="18"/>
+      <c r="B2171" s="18">
+        <v>45930</v>
+      </c>
       <c r="C2171" s="1"/>
       <c r="D2171" s="1"/>
       <c r="E2171" s="1">
         <f t="shared" si="37"/>
         <v>0</v>
       </c>
-      <c r="F2171" s="1"/>
-      <c r="G2171" s="10"/>
-      <c r="H2171" s="3"/>
-      <c r="I2171" s="12"/>
-      <c r="J2171" s="7"/>
-      <c r="K2171" s="7"/>
+      <c r="F2171" s="1">
+        <v>133.28</v>
+      </c>
+      <c r="G2171" s="10">
+        <v>838.35</v>
+      </c>
+      <c r="H2171" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2171" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2171" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2171" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2172" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2172" s="18">
@@ -71171,13 +71537,31 @@
       </c>
     </row>
     <row r="2181" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2181" s="17"/>
+      <c r="B2181" s="17">
+        <v>45937</v>
+      </c>
       <c r="E2181" s="1">
         <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="G2181" s="13"/>
-      <c r="I2181" s="12"/>
+      <c r="F2181" s="2">
+        <v>134.22800000000001</v>
+      </c>
+      <c r="G2181" s="13">
+        <v>781.2</v>
+      </c>
+      <c r="H2181" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2181" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2181" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2181" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2182" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2182" s="17">
@@ -71407,19 +71791,33 @@
       </c>
     </row>
     <row r="2189" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2189" s="18"/>
+      <c r="B2189" s="18">
+        <v>45932</v>
+      </c>
       <c r="C2189" s="1"/>
       <c r="D2189" s="1"/>
       <c r="E2189" s="1">
         <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="F2189" s="1"/>
-      <c r="G2189" s="10"/>
-      <c r="H2189" s="3"/>
-      <c r="I2189" s="12"/>
-      <c r="J2189" s="7"/>
-      <c r="K2189" s="7"/>
+      <c r="F2189" s="1">
+        <v>140</v>
+      </c>
+      <c r="G2189" s="10">
+        <v>824.6</v>
+      </c>
+      <c r="H2189" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2189" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2189" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="K2189" s="7" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2190" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2190" s="18">
@@ -71451,19 +71849,33 @@
       </c>
     </row>
     <row r="2191" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2191" s="18"/>
+      <c r="B2191" s="18">
+        <v>45943</v>
+      </c>
       <c r="C2191" s="1"/>
       <c r="D2191" s="1"/>
       <c r="E2191" s="1">
         <f t="shared" si="38"/>
         <v>0</v>
       </c>
-      <c r="F2191" s="1"/>
-      <c r="G2191" s="10"/>
-      <c r="H2191" s="3"/>
-      <c r="I2191" s="12"/>
-      <c r="J2191" s="7"/>
-      <c r="K2191" s="7"/>
+      <c r="F2191" s="1">
+        <v>120.73699999999999</v>
+      </c>
+      <c r="G2191" s="10">
+        <v>702.68</v>
+      </c>
+      <c r="H2191" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2191" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2191" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2191" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="2192" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2192" s="18">
@@ -77579,94 +77991,178 @@
       </c>
     </row>
     <row r="2376" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2376" s="18"/>
+      <c r="B2376" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2376" s="1"/>
       <c r="D2376" s="1"/>
       <c r="E2376" s="1">
         <f>D2376-C2376</f>
         <v>0</v>
       </c>
-      <c r="F2376" s="1"/>
-      <c r="G2376" s="10"/>
-      <c r="H2376" s="3"/>
-      <c r="I2376" s="12"/>
-      <c r="J2376" s="7"/>
-      <c r="K2376" s="7"/>
+      <c r="F2376" s="1">
+        <v>508.02699999999999</v>
+      </c>
+      <c r="G2376" s="10">
+        <v>2956.72</v>
+      </c>
+      <c r="H2376" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2376" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2376" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2376" s="7" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="2377" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2377" s="18"/>
+      <c r="B2377" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2377" s="1"/>
       <c r="D2377" s="1"/>
       <c r="E2377" s="1">
         <f>D2377-C2377</f>
         <v>0</v>
       </c>
-      <c r="F2377" s="1"/>
-      <c r="G2377" s="10"/>
-      <c r="H2377" s="3"/>
-      <c r="I2377" s="12"/>
-      <c r="J2377" s="7"/>
-      <c r="K2377" s="7"/>
+      <c r="F2377" s="1">
+        <v>101.80200000000001</v>
+      </c>
+      <c r="G2377" s="10">
+        <v>592.48</v>
+      </c>
+      <c r="H2377" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2377" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2377" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2377" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="2378" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2378" s="18"/>
+      <c r="B2378" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2378" s="1"/>
       <c r="D2378" s="1"/>
       <c r="E2378" s="1">
         <f>D2378-C2378</f>
         <v>0</v>
       </c>
-      <c r="F2378" s="1"/>
-      <c r="G2378" s="10"/>
-      <c r="H2378" s="3"/>
-      <c r="I2378" s="12"/>
-      <c r="J2378" s="7"/>
-      <c r="K2378" s="7"/>
+      <c r="F2378" s="1">
+        <v>127.41</v>
+      </c>
+      <c r="G2378" s="10">
+        <v>814.15</v>
+      </c>
+      <c r="H2378" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2378" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2378" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="K2378" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2379" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2379" s="18"/>
+      <c r="B2379" s="18">
+        <v>45924</v>
+      </c>
       <c r="C2379" s="1"/>
       <c r="D2379" s="1"/>
       <c r="E2379" s="1">
         <f>D2379-C2379</f>
         <v>0</v>
       </c>
-      <c r="F2379" s="1"/>
-      <c r="G2379" s="10"/>
-      <c r="H2379" s="3"/>
-      <c r="I2379" s="12"/>
-      <c r="J2379" s="7"/>
-      <c r="K2379" s="7"/>
+      <c r="F2379" s="1">
+        <v>12.39</v>
+      </c>
+      <c r="G2379" s="10">
+        <v>70.5</v>
+      </c>
+      <c r="H2379" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2379" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2379" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2379" s="7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="2380" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2380" s="18"/>
+      <c r="B2380" s="18">
+        <v>45938</v>
+      </c>
       <c r="C2380" s="1"/>
       <c r="D2380" s="1"/>
       <c r="E2380" s="1">
         <f>D2380-C2380</f>
         <v>0</v>
       </c>
-      <c r="F2380" s="1"/>
-      <c r="G2380" s="10"/>
-      <c r="H2380" s="3"/>
-      <c r="I2380" s="12"/>
-      <c r="J2380" s="7"/>
-      <c r="K2380" s="7"/>
+      <c r="F2380" s="1">
+        <v>199.68</v>
+      </c>
+      <c r="G2380" s="10">
+        <v>1248.03</v>
+      </c>
+      <c r="H2380" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2380" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2380" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="K2380" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2381" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2381" s="18"/>
+      <c r="B2381" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2381" s="1"/>
       <c r="D2381" s="1"/>
       <c r="E2381" s="1">
         <f t="shared" ref="E2381:E2444" si="42">D2381-C2381</f>
         <v>0</v>
       </c>
-      <c r="F2381" s="1"/>
-      <c r="G2381" s="10"/>
-      <c r="H2381" s="3"/>
-      <c r="I2381" s="12"/>
-      <c r="J2381" s="7"/>
-      <c r="K2381" s="7"/>
+      <c r="F2381" s="1">
+        <v>62.360999999999997</v>
+      </c>
+      <c r="G2381" s="10">
+        <v>362.94</v>
+      </c>
+      <c r="H2381" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2381" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2381" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2381" s="7" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="2382" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2382" s="18">
@@ -77727,34 +78223,62 @@
       </c>
     </row>
     <row r="2384" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2384" s="18"/>
+      <c r="B2384" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2384" s="1"/>
       <c r="D2384" s="1"/>
       <c r="E2384" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2384" s="1"/>
-      <c r="G2384" s="10"/>
-      <c r="H2384" s="3"/>
-      <c r="I2384" s="12"/>
-      <c r="J2384" s="7"/>
-      <c r="K2384" s="7"/>
+      <c r="F2384" s="1">
+        <v>49.673000000000002</v>
+      </c>
+      <c r="G2384" s="10">
+        <v>289.10000000000002</v>
+      </c>
+      <c r="H2384" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2384" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2384" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2384" s="7" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="2385" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2385" s="18"/>
+      <c r="B2385" s="18">
+        <v>45936</v>
+      </c>
       <c r="C2385" s="1"/>
       <c r="D2385" s="1"/>
       <c r="E2385" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2385" s="1"/>
-      <c r="G2385" s="10"/>
-      <c r="H2385" s="3"/>
-      <c r="I2385" s="12"/>
-      <c r="J2385" s="7"/>
-      <c r="K2385" s="7"/>
+      <c r="F2385" s="1">
+        <v>189.96700000000001</v>
+      </c>
+      <c r="G2385" s="10">
+        <v>1105.6099999999999</v>
+      </c>
+      <c r="H2385" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2385" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2385" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2385" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="2386" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2386" s="18">
@@ -77786,19 +78310,33 @@
       </c>
     </row>
     <row r="2387" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2387" s="18"/>
+      <c r="B2387" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2387" s="1"/>
       <c r="D2387" s="1"/>
       <c r="E2387" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2387" s="1"/>
-      <c r="G2387" s="10"/>
-      <c r="H2387" s="3"/>
-      <c r="I2387" s="12"/>
-      <c r="J2387" s="7"/>
-      <c r="K2387" s="7"/>
+      <c r="F2387" s="1">
+        <v>158.68</v>
+      </c>
+      <c r="G2387" s="10">
+        <v>998.14</v>
+      </c>
+      <c r="H2387" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2387" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2387" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2387" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="2388" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2388" s="18">
@@ -77830,19 +78368,33 @@
       </c>
     </row>
     <row r="2389" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2389" s="18"/>
+      <c r="B2389" s="18">
+        <v>45924</v>
+      </c>
       <c r="C2389" s="1"/>
       <c r="D2389" s="1"/>
       <c r="E2389" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2389" s="1"/>
-      <c r="G2389" s="10"/>
-      <c r="H2389" s="3"/>
-      <c r="I2389" s="12"/>
-      <c r="J2389" s="7"/>
-      <c r="K2389" s="7"/>
+      <c r="F2389" s="1">
+        <v>22.91</v>
+      </c>
+      <c r="G2389" s="10">
+        <v>1395.59</v>
+      </c>
+      <c r="H2389" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2389" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2389" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2389" s="7" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="2390" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2390" s="18">
@@ -77932,49 +78484,91 @@
       </c>
     </row>
     <row r="2393" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2393" s="18"/>
+      <c r="B2393" s="18">
+        <v>45943</v>
+      </c>
       <c r="C2393" s="1"/>
       <c r="D2393" s="1"/>
       <c r="E2393" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2393" s="1"/>
-      <c r="G2393" s="10"/>
-      <c r="H2393" s="3"/>
-      <c r="I2393" s="12"/>
-      <c r="J2393" s="7"/>
-      <c r="K2393" s="7"/>
+      <c r="F2393" s="1">
+        <v>197.18</v>
+      </c>
+      <c r="G2393" s="10">
+        <v>1240.27</v>
+      </c>
+      <c r="H2393" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2393" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2393" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2393" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2394" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2394" s="18"/>
+      <c r="B2394" s="18">
+        <v>45936</v>
+      </c>
       <c r="C2394" s="1"/>
       <c r="D2394" s="1"/>
       <c r="E2394" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2394" s="1"/>
-      <c r="G2394" s="10"/>
-      <c r="H2394" s="3"/>
-      <c r="I2394" s="12"/>
-      <c r="J2394" s="7"/>
-      <c r="K2394" s="7"/>
+      <c r="F2394" s="1">
+        <v>212.91</v>
+      </c>
+      <c r="G2394" s="10">
+        <v>1339.21</v>
+      </c>
+      <c r="H2394" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2394" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2394" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2394" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2395" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2395" s="18"/>
+      <c r="B2395" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2395" s="1"/>
       <c r="D2395" s="1"/>
       <c r="E2395" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2395" s="1"/>
-      <c r="G2395" s="10"/>
-      <c r="H2395" s="3"/>
-      <c r="I2395" s="12"/>
-      <c r="J2395" s="7"/>
-      <c r="K2395" s="7"/>
+      <c r="F2395" s="1">
+        <v>135.13</v>
+      </c>
+      <c r="G2395" s="10">
+        <v>816.19</v>
+      </c>
+      <c r="H2395" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2395" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2395" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2395" s="7" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="2396" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2396" s="18"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-14 14:10
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="641" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5571D5BF-7362-4C43-BC82-CBB6A8D3CA90}"/>
+  <xr:revisionPtr revIDLastSave="764" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CECC443E-7596-4BE7-941F-214DFCA73E83}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8066" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8104" uniqueCount="337">
   <si>
     <t>Data</t>
   </si>
@@ -1045,6 +1045,12 @@
   <si>
     <t>POSTO SOARES</t>
   </si>
+  <si>
+    <t>Diesel s10</t>
+  </si>
+  <si>
+    <t>POSTO RABELO</t>
+  </si>
 </sst>
 </file>
 
@@ -78571,94 +78577,176 @@
       </c>
     </row>
     <row r="2396" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2396" s="18"/>
+      <c r="B2396" s="18">
+        <v>45939</v>
+      </c>
       <c r="C2396" s="1"/>
       <c r="D2396" s="1"/>
       <c r="E2396" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2396" s="1"/>
-      <c r="G2396" s="10"/>
-      <c r="H2396" s="3"/>
-      <c r="I2396" s="12"/>
-      <c r="J2396" s="7"/>
-      <c r="K2396" s="7"/>
+      <c r="F2396" s="1">
+        <v>344.37</v>
+      </c>
+      <c r="G2396" s="10">
+        <v>2166.1</v>
+      </c>
+      <c r="H2396" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2396" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2396" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2396" s="7" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="2397" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2397" s="18"/>
+      <c r="B2397" s="18">
+        <v>45936</v>
+      </c>
       <c r="C2397" s="1"/>
       <c r="D2397" s="1"/>
       <c r="E2397" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2397" s="1"/>
-      <c r="G2397" s="10"/>
-      <c r="H2397" s="3"/>
-      <c r="I2397" s="12"/>
-      <c r="J2397" s="7"/>
+      <c r="F2397" s="1">
+        <v>235.03</v>
+      </c>
+      <c r="G2397" s="10">
+        <v>1478.33</v>
+      </c>
+      <c r="H2397" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2397" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2397" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="K2397" s="7"/>
     </row>
     <row r="2398" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2398" s="18"/>
+      <c r="B2398" s="18">
+        <v>45932</v>
+      </c>
       <c r="C2398" s="1"/>
       <c r="D2398" s="1"/>
       <c r="E2398" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2398" s="1"/>
-      <c r="G2398" s="10"/>
-      <c r="H2398" s="3"/>
-      <c r="I2398" s="12"/>
-      <c r="J2398" s="7"/>
-      <c r="K2398" s="7"/>
+      <c r="F2398" s="1">
+        <v>202</v>
+      </c>
+      <c r="G2398" s="10">
+        <v>1220.08</v>
+      </c>
+      <c r="H2398" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2398" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2398" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="K2398" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2399" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2399" s="18"/>
+      <c r="B2399" s="18">
+        <v>45933</v>
+      </c>
       <c r="C2399" s="1"/>
       <c r="D2399" s="1"/>
       <c r="E2399" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2399" s="1"/>
-      <c r="G2399" s="10"/>
-      <c r="H2399" s="3"/>
-      <c r="I2399" s="12"/>
-      <c r="J2399" s="7"/>
-      <c r="K2399" s="7"/>
+      <c r="F2399" s="1">
+        <v>79.489999999999995</v>
+      </c>
+      <c r="G2399" s="10">
+        <v>500</v>
+      </c>
+      <c r="H2399" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="I2399" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2399" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2399" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2400" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2400" s="18"/>
+      <c r="B2400" s="18">
+        <v>45932</v>
+      </c>
       <c r="C2400" s="1"/>
       <c r="D2400" s="1"/>
       <c r="E2400" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2400" s="1"/>
-      <c r="G2400" s="10"/>
-      <c r="H2400" s="3"/>
-      <c r="I2400" s="12"/>
-      <c r="J2400" s="7"/>
-      <c r="K2400" s="7"/>
+      <c r="F2400" s="1">
+        <v>103.99</v>
+      </c>
+      <c r="G2400" s="10">
+        <v>664.5</v>
+      </c>
+      <c r="H2400" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2400" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2400" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="K2400" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2401" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2401" s="18"/>
+      <c r="B2401" s="18">
+        <v>45931</v>
+      </c>
       <c r="C2401" s="1"/>
       <c r="D2401" s="1"/>
       <c r="E2401" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2401" s="1"/>
-      <c r="G2401" s="10"/>
-      <c r="H2401" s="3"/>
-      <c r="I2401" s="12"/>
-      <c r="J2401" s="7"/>
-      <c r="K2401" s="7"/>
+      <c r="F2401" s="1">
+        <v>200.33699999999999</v>
+      </c>
+      <c r="G2401" s="10">
+        <v>1200.02</v>
+      </c>
+      <c r="H2401" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2401" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2401" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="K2401" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="2402" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2402" s="18">
@@ -78690,33 +78778,62 @@
       </c>
     </row>
     <row r="2403" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2403" s="18"/>
+      <c r="B2403" s="18">
+        <v>45933</v>
+      </c>
       <c r="C2403" s="1"/>
       <c r="D2403" s="1"/>
       <c r="E2403" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2403" s="1"/>
-      <c r="G2403" s="10"/>
-      <c r="H2403" s="3"/>
-      <c r="I2403" s="12"/>
-      <c r="J2403" s="7"/>
-      <c r="K2403" s="7"/>
+      <c r="F2403" s="1">
+        <v>54.186</v>
+      </c>
+      <c r="G2403" s="10">
+        <v>315.36</v>
+      </c>
+      <c r="H2403" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2403" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2403" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2403" s="7" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="2404" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2404" s="18"/>
+      <c r="B2404" s="18">
+        <v>45933</v>
+      </c>
       <c r="C2404" s="1"/>
       <c r="D2404" s="1"/>
       <c r="E2404" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2404" s="1"/>
-      <c r="G2404" s="10"/>
-      <c r="H2404" s="3"/>
-      <c r="J2404" s="7"/>
-      <c r="K2404" s="7"/>
+      <c r="F2404" s="1">
+        <v>86.747</v>
+      </c>
+      <c r="G2404" s="10">
+        <v>504.86</v>
+      </c>
+      <c r="H2404" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2404" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2404" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2404" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="2405" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2405" s="17">
@@ -79055,18 +79172,33 @@
       </c>
     </row>
     <row r="2415" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2415" s="18"/>
+      <c r="B2415" s="18">
+        <v>45932</v>
+      </c>
       <c r="C2415" s="1"/>
       <c r="D2415" s="1"/>
       <c r="E2415" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2415" s="1"/>
-      <c r="G2415" s="10"/>
-      <c r="H2415" s="3"/>
-      <c r="J2415" s="7"/>
-      <c r="K2415" s="7"/>
+      <c r="F2415" s="1">
+        <v>41.72</v>
+      </c>
+      <c r="G2415" s="10">
+        <v>249.53</v>
+      </c>
+      <c r="H2415" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2415" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2415" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2415" s="7" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="2416" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2416" s="17">
@@ -79342,32 +79474,62 @@
       </c>
     </row>
     <row r="2425" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2425" s="18"/>
+      <c r="B2425" s="18">
+        <v>45933</v>
+      </c>
       <c r="C2425" s="1"/>
       <c r="D2425" s="1"/>
       <c r="E2425" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2425" s="1"/>
-      <c r="G2425" s="10"/>
-      <c r="H2425" s="3"/>
-      <c r="J2425" s="7"/>
-      <c r="K2425" s="7"/>
+      <c r="F2425" s="1">
+        <v>121.97499999999999</v>
+      </c>
+      <c r="G2425" s="10">
+        <v>709.89</v>
+      </c>
+      <c r="H2425" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2425" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2425" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2425" s="7" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="2426" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2426" s="18"/>
+      <c r="B2426" s="18">
+        <v>45936</v>
+      </c>
       <c r="C2426" s="1"/>
       <c r="D2426" s="1"/>
       <c r="E2426" s="1">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="F2426" s="1"/>
-      <c r="G2426" s="10"/>
-      <c r="H2426" s="3"/>
-      <c r="J2426" s="7"/>
-      <c r="K2426" s="7"/>
+      <c r="F2426" s="1">
+        <v>200.28</v>
+      </c>
+      <c r="G2426" s="10">
+        <v>1259.76</v>
+      </c>
+      <c r="H2426" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2426" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2426" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2426" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="2427" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2427" s="17">
@@ -80455,32 +80617,62 @@
       </c>
     </row>
     <row r="2462" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2462" s="18"/>
+      <c r="B2462" s="18">
+        <v>45937</v>
+      </c>
       <c r="C2462" s="1"/>
       <c r="D2462" s="1"/>
       <c r="E2462" s="1">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F2462" s="1"/>
-      <c r="G2462" s="10"/>
-      <c r="H2462" s="3"/>
-      <c r="J2462" s="7"/>
-      <c r="K2462" s="7"/>
+      <c r="F2462" s="1">
+        <v>169.12</v>
+      </c>
+      <c r="G2462" s="10">
+        <v>1063.8</v>
+      </c>
+      <c r="H2462" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2462" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2462" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2462" s="7" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="2463" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2463" s="18"/>
+      <c r="B2463" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2463" s="1"/>
       <c r="D2463" s="1"/>
       <c r="E2463" s="1">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F2463" s="1"/>
-      <c r="G2463" s="10"/>
-      <c r="H2463" s="3"/>
-      <c r="J2463" s="7"/>
-      <c r="K2463" s="7"/>
+      <c r="F2463" s="1">
+        <v>108.66</v>
+      </c>
+      <c r="G2463" s="10">
+        <v>632.4</v>
+      </c>
+      <c r="H2463" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2463" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2463" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2463" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="2464" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2464" s="18"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-14 16:32
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="764" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CECC443E-7596-4BE7-941F-214DFCA73E83}"/>
+  <xr:revisionPtr revIDLastSave="788" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFB4641F-19E1-4630-9815-B07BC92CBD98}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8104" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8113" uniqueCount="337">
   <si>
     <t>Data</t>
   </si>
@@ -80675,18 +80675,33 @@
       </c>
     </row>
     <row r="2464" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2464" s="18"/>
+      <c r="B2464" s="18">
+        <v>45944</v>
+      </c>
       <c r="C2464" s="1"/>
       <c r="D2464" s="1"/>
       <c r="E2464" s="1">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F2464" s="1"/>
-      <c r="G2464" s="10"/>
-      <c r="H2464" s="3"/>
-      <c r="J2464" s="7"/>
-      <c r="K2464" s="7"/>
+      <c r="F2464" s="1">
+        <v>129.077</v>
+      </c>
+      <c r="G2464" s="10">
+        <v>751.23</v>
+      </c>
+      <c r="H2464" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2464" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2464" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2464" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="2465" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2465" s="17">
@@ -80929,18 +80944,33 @@
       </c>
     </row>
     <row r="2472" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2472" s="18"/>
+      <c r="B2472" s="18">
+        <v>45944</v>
+      </c>
       <c r="C2472" s="1"/>
       <c r="D2472" s="1"/>
       <c r="E2472" s="1">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F2472" s="1"/>
-      <c r="G2472" s="10"/>
-      <c r="H2472" s="3"/>
-      <c r="J2472" s="7"/>
-      <c r="K2472" s="7"/>
+      <c r="F2472" s="1">
+        <v>207.83199999999999</v>
+      </c>
+      <c r="G2472" s="10">
+        <v>1209.58</v>
+      </c>
+      <c r="H2472" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2472" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2472" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2472" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2473" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2473" s="17">
@@ -81150,18 +81180,33 @@
       <c r="K2481" s="7"/>
     </row>
     <row r="2482" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2482" s="18"/>
+      <c r="B2482" s="18">
+        <v>45940</v>
+      </c>
       <c r="C2482" s="1"/>
       <c r="D2482" s="1"/>
       <c r="E2482" s="1">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F2482" s="1"/>
-      <c r="G2482" s="10"/>
-      <c r="H2482" s="3"/>
-      <c r="J2482" s="7"/>
-      <c r="K2482" s="7"/>
+      <c r="F2482" s="1">
+        <v>143.72999999999999</v>
+      </c>
+      <c r="G2482" s="10">
+        <v>932.81</v>
+      </c>
+      <c r="H2482" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2482" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2482" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2482" s="7" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="2483" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2483" s="18"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-15 16:34
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="863" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FCAAA74-9836-4815-9EF5-12861ADC22C0}"/>
+  <xr:revisionPtr revIDLastSave="864" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3E31DDF-85EC-4B78-A3A1-A93CD8E71BE4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -1595,7 +1595,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-  <sheetPr filterMode="1"/>
   <dimension ref="B1:L2851"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -81429,7 +81428,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2483" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2483" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2483" s="18"/>
       <c r="C2483" s="1"/>
       <c r="D2483" s="1"/>
@@ -82190,7 +82189,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="2507" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2507" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2507" s="18"/>
       <c r="C2507" s="1"/>
       <c r="D2507" s="1"/>
@@ -82204,7 +82203,7 @@
       <c r="J2507" s="7"/>
       <c r="K2507" s="7"/>
     </row>
-    <row r="2508" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2508" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2508" s="18"/>
       <c r="C2508" s="1"/>
       <c r="D2508" s="1"/>
@@ -82218,7 +82217,7 @@
       <c r="J2508" s="7"/>
       <c r="K2508" s="7"/>
     </row>
-    <row r="2509" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2509" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2509" s="18"/>
       <c r="C2509" s="1"/>
       <c r="D2509" s="1"/>
@@ -82232,7 +82231,7 @@
       <c r="J2509" s="7"/>
       <c r="K2509" s="7"/>
     </row>
-    <row r="2510" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2510" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2510" s="18"/>
       <c r="C2510" s="1"/>
       <c r="D2510" s="1"/>
@@ -82738,7 +82737,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2526" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2526" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2526" s="18"/>
       <c r="C2526" s="1"/>
       <c r="D2526" s="1"/>
@@ -82752,7 +82751,7 @@
       <c r="J2526" s="7"/>
       <c r="K2526" s="7"/>
     </row>
-    <row r="2527" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2527" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2527" s="18"/>
       <c r="C2527" s="1"/>
       <c r="D2527" s="1"/>
@@ -82766,7 +82765,7 @@
       <c r="J2527" s="7"/>
       <c r="K2527" s="7"/>
     </row>
-    <row r="2528" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2528" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2528" s="18"/>
       <c r="C2528" s="1"/>
       <c r="D2528" s="1"/>
@@ -82780,7 +82779,7 @@
       <c r="J2528" s="7"/>
       <c r="K2528" s="7"/>
     </row>
-    <row r="2529" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2529" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2529" s="18"/>
       <c r="C2529" s="1"/>
       <c r="D2529" s="1"/>
@@ -82794,7 +82793,7 @@
       <c r="J2529" s="7"/>
       <c r="K2529" s="7"/>
     </row>
-    <row r="2530" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2530" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2530" s="18"/>
       <c r="C2530" s="1"/>
       <c r="D2530" s="1"/>
@@ -82808,7 +82807,7 @@
       <c r="J2530" s="7"/>
       <c r="K2530" s="7"/>
     </row>
-    <row r="2531" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2531" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2531" s="18"/>
       <c r="C2531" s="1"/>
       <c r="D2531" s="1"/>
@@ -83191,7 +83190,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="2543" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2543" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2543" s="18"/>
       <c r="C2543" s="1"/>
       <c r="D2543" s="1"/>
@@ -83205,7 +83204,7 @@
       <c r="J2543" s="7"/>
       <c r="K2543" s="7"/>
     </row>
-    <row r="2544" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2544" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2544" s="18"/>
       <c r="C2544" s="1"/>
       <c r="D2544" s="1"/>
@@ -83219,7 +83218,7 @@
       <c r="J2544" s="7"/>
       <c r="K2544" s="7"/>
     </row>
-    <row r="2545" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2545" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2545" s="18"/>
       <c r="C2545" s="1"/>
       <c r="D2545" s="1"/>
@@ -83233,7 +83232,7 @@
       <c r="J2545" s="7"/>
       <c r="K2545" s="7"/>
     </row>
-    <row r="2546" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2546" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2546" s="18"/>
       <c r="C2546" s="1"/>
       <c r="D2546" s="1"/>
@@ -83247,7 +83246,7 @@
       <c r="J2546" s="7"/>
       <c r="K2546" s="7"/>
     </row>
-    <row r="2547" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2547" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2547" s="18"/>
       <c r="C2547" s="1"/>
       <c r="D2547" s="1"/>
@@ -83261,7 +83260,7 @@
       <c r="J2547" s="7"/>
       <c r="K2547" s="7"/>
     </row>
-    <row r="2548" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2548" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2548" s="18"/>
       <c r="C2548" s="1"/>
       <c r="D2548" s="1"/>
@@ -83311,7 +83310,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="2550" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2550" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2550" s="17"/>
       <c r="E2550" s="1">
         <f t="shared" si="44"/>
@@ -83580,7 +83579,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2559" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2559" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2559" s="18"/>
       <c r="C2559" s="1"/>
       <c r="D2559" s="1"/>
@@ -83594,7 +83593,7 @@
       <c r="J2559" s="7"/>
       <c r="K2559" s="7"/>
     </row>
-    <row r="2560" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2560" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2560" s="18"/>
       <c r="C2560" s="1"/>
       <c r="D2560" s="1"/>
@@ -84838,7 +84837,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2598" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2598" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2598" s="18"/>
       <c r="C2598" s="1"/>
       <c r="D2598" s="1"/>
@@ -84852,7 +84851,7 @@
       <c r="J2598" s="7"/>
       <c r="K2598" s="7"/>
     </row>
-    <row r="2599" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2599" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2599" s="18"/>
       <c r="C2599" s="1"/>
       <c r="D2599" s="1"/>
@@ -84866,7 +84865,7 @@
       <c r="J2599" s="7"/>
       <c r="K2599" s="7"/>
     </row>
-    <row r="2600" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2600" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2600" s="18"/>
       <c r="C2600" s="1"/>
       <c r="D2600" s="1"/>
@@ -85174,7 +85173,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="2610" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2610" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2610" s="18"/>
       <c r="C2610" s="1"/>
       <c r="D2610" s="1"/>
@@ -85188,7 +85187,7 @@
       <c r="J2610" s="7"/>
       <c r="K2610" s="7"/>
     </row>
-    <row r="2611" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2611" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2611" s="18"/>
       <c r="C2611" s="1"/>
       <c r="D2611" s="1"/>
@@ -85202,7 +85201,7 @@
       <c r="J2611" s="7"/>
       <c r="K2611" s="7"/>
     </row>
-    <row r="2612" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2612" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2612" s="18"/>
       <c r="C2612" s="1"/>
       <c r="D2612" s="1"/>
@@ -85216,7 +85215,7 @@
       <c r="J2612" s="7"/>
       <c r="K2612" s="7"/>
     </row>
-    <row r="2613" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2613" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2613" s="18"/>
       <c r="C2613" s="1"/>
       <c r="D2613" s="1"/>
@@ -85707,7 +85706,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="2628" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2628" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2628" s="18"/>
       <c r="C2628" s="1"/>
       <c r="D2628" s="1"/>
@@ -85721,7 +85720,7 @@
       <c r="J2628" s="7"/>
       <c r="K2628" s="7"/>
     </row>
-    <row r="2629" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2629" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2629" s="18"/>
       <c r="C2629" s="1"/>
       <c r="D2629" s="1"/>
@@ -85735,7 +85734,7 @@
       <c r="J2629" s="7"/>
       <c r="K2629" s="7"/>
     </row>
-    <row r="2630" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2630" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2630" s="18"/>
       <c r="C2630" s="1"/>
       <c r="D2630" s="1"/>
@@ -85749,7 +85748,7 @@
       <c r="J2630" s="7"/>
       <c r="K2630" s="7"/>
     </row>
-    <row r="2631" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2631" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2631" s="18"/>
       <c r="C2631" s="1"/>
       <c r="D2631" s="1"/>
@@ -85763,7 +85762,7 @@
       <c r="J2631" s="7"/>
       <c r="K2631" s="7"/>
     </row>
-    <row r="2632" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2632" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2632" s="18"/>
       <c r="C2632" s="1"/>
       <c r="D2632" s="1"/>
@@ -85777,7 +85776,7 @@
       <c r="J2632" s="7"/>
       <c r="K2632" s="7"/>
     </row>
-    <row r="2633" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2633" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2633" s="18"/>
       <c r="C2633" s="1"/>
       <c r="D2633" s="1"/>
@@ -86337,7 +86336,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2650" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2650" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2650" s="18"/>
       <c r="C2650" s="1"/>
       <c r="D2650" s="1"/>
@@ -86351,7 +86350,7 @@
       <c r="J2650" s="7"/>
       <c r="K2650" s="7"/>
     </row>
-    <row r="2651" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2651" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2651" s="18"/>
       <c r="C2651" s="1"/>
       <c r="D2651" s="1"/>
@@ -86365,7 +86364,7 @@
       <c r="J2651" s="7"/>
       <c r="K2651" s="7"/>
     </row>
-    <row r="2652" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2652" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2652" s="18"/>
       <c r="C2652" s="1"/>
       <c r="D2652" s="1"/>
@@ -86379,7 +86378,7 @@
       <c r="J2652" s="7"/>
       <c r="K2652" s="7"/>
     </row>
-    <row r="2653" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2653" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2653" s="18"/>
       <c r="C2653" s="1"/>
       <c r="D2653" s="1"/>
@@ -86393,7 +86392,7 @@
       <c r="J2653" s="7"/>
       <c r="K2653" s="7"/>
     </row>
-    <row r="2654" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2654" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2654" s="18"/>
       <c r="C2654" s="1"/>
       <c r="D2654" s="1"/>
@@ -86773,7 +86772,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="2666" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2666" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2666" s="18"/>
       <c r="C2666" s="1"/>
       <c r="D2666" s="1"/>
@@ -86787,7 +86786,7 @@
       <c r="J2666" s="7"/>
       <c r="K2666" s="7"/>
     </row>
-    <row r="2667" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2667" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2667" s="18"/>
       <c r="C2667" s="1"/>
       <c r="D2667" s="1"/>
@@ -86801,7 +86800,7 @@
       <c r="J2667" s="7"/>
       <c r="K2667" s="7"/>
     </row>
-    <row r="2668" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2668" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2668" s="18"/>
       <c r="C2668" s="1"/>
       <c r="D2668" s="1"/>
@@ -86815,7 +86814,7 @@
       <c r="J2668" s="7"/>
       <c r="K2668" s="7"/>
     </row>
-    <row r="2669" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2669" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2669" s="18"/>
       <c r="C2669" s="1"/>
       <c r="D2669" s="1"/>
@@ -86829,7 +86828,7 @@
       <c r="J2669" s="7"/>
       <c r="K2669" s="7"/>
     </row>
-    <row r="2670" spans="2:12" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2670" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2670" s="18"/>
       <c r="C2670" s="1"/>
       <c r="D2670" s="1"/>
@@ -87476,7 +87475,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2690" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2690" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2690" s="18"/>
       <c r="C2690" s="1"/>
       <c r="D2690" s="1"/>
@@ -87488,7 +87487,7 @@
       <c r="G2690" s="10"/>
       <c r="K2690" s="7"/>
     </row>
-    <row r="2691" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2691" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2691" s="18"/>
       <c r="C2691" s="1"/>
       <c r="D2691" s="1"/>
@@ -87500,7 +87499,7 @@
       <c r="G2691" s="10"/>
       <c r="K2691" s="7"/>
     </row>
-    <row r="2692" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2692" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2692" s="18"/>
       <c r="C2692" s="1"/>
       <c r="D2692" s="1"/>
@@ -87512,7 +87511,7 @@
       <c r="G2692" s="10"/>
       <c r="K2692" s="7"/>
     </row>
-    <row r="2693" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2693" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2693" s="18"/>
       <c r="C2693" s="1"/>
       <c r="D2693" s="1"/>
@@ -87524,7 +87523,7 @@
       <c r="G2693" s="10"/>
       <c r="K2693" s="7"/>
     </row>
-    <row r="2694" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2694" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2694" s="18"/>
       <c r="C2694" s="1"/>
       <c r="D2694" s="1"/>
@@ -87536,7 +87535,7 @@
       <c r="G2694" s="10"/>
       <c r="K2694" s="7"/>
     </row>
-    <row r="2695" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2695" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2695" s="18"/>
       <c r="C2695" s="1"/>
       <c r="D2695" s="1"/>
@@ -87548,7 +87547,7 @@
       <c r="G2695" s="10"/>
       <c r="K2695" s="7"/>
     </row>
-    <row r="2696" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2696" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2696" s="18"/>
       <c r="C2696" s="1"/>
       <c r="D2696" s="1"/>
@@ -87560,7 +87559,7 @@
       <c r="G2696" s="10"/>
       <c r="K2696" s="7"/>
     </row>
-    <row r="2697" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2697" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2697" s="18"/>
       <c r="C2697" s="1"/>
       <c r="D2697" s="1"/>
@@ -87572,7 +87571,7 @@
       <c r="G2697" s="10"/>
       <c r="K2697" s="7"/>
     </row>
-    <row r="2698" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2698" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2698" s="18"/>
       <c r="C2698" s="1"/>
       <c r="D2698" s="1"/>
@@ -87584,7 +87583,7 @@
       <c r="G2698" s="10"/>
       <c r="K2698" s="7"/>
     </row>
-    <row r="2699" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2699" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2699" s="18"/>
       <c r="C2699" s="1"/>
       <c r="D2699" s="1"/>
@@ -87596,7 +87595,7 @@
       <c r="G2699" s="10"/>
       <c r="K2699" s="7"/>
     </row>
-    <row r="2700" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2700" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2700" s="18"/>
       <c r="C2700" s="1"/>
       <c r="D2700" s="1"/>
@@ -87608,7 +87607,7 @@
       <c r="G2700" s="10"/>
       <c r="K2700" s="7"/>
     </row>
-    <row r="2701" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2701" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2701" s="18"/>
       <c r="C2701" s="1"/>
       <c r="D2701" s="1"/>
@@ -87620,7 +87619,7 @@
       <c r="G2701" s="10"/>
       <c r="K2701" s="7"/>
     </row>
-    <row r="2702" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2702" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2702" s="18"/>
       <c r="C2702" s="1"/>
       <c r="D2702" s="1"/>
@@ -87632,7 +87631,7 @@
       <c r="G2702" s="10"/>
       <c r="K2702" s="7"/>
     </row>
-    <row r="2703" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2703" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2703" s="18"/>
       <c r="C2703" s="1"/>
       <c r="D2703" s="1"/>
@@ -87644,7 +87643,7 @@
       <c r="G2703" s="10"/>
       <c r="K2703" s="7"/>
     </row>
-    <row r="2704" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2704" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2704" s="18"/>
       <c r="C2704" s="1"/>
       <c r="D2704" s="1"/>
@@ -87656,7 +87655,7 @@
       <c r="G2704" s="10"/>
       <c r="K2704" s="7"/>
     </row>
-    <row r="2705" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2705" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2705" s="18"/>
       <c r="C2705" s="1"/>
       <c r="D2705" s="1"/>
@@ -87668,7 +87667,7 @@
       <c r="G2705" s="10"/>
       <c r="K2705" s="7"/>
     </row>
-    <row r="2706" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2706" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2706" s="18"/>
       <c r="C2706" s="1"/>
       <c r="D2706" s="1"/>
@@ -87680,7 +87679,7 @@
       <c r="G2706" s="10"/>
       <c r="K2706" s="7"/>
     </row>
-    <row r="2707" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2707" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2707" s="18"/>
       <c r="C2707" s="1"/>
       <c r="D2707" s="1"/>
@@ -87692,7 +87691,7 @@
       <c r="G2707" s="10"/>
       <c r="K2707" s="7"/>
     </row>
-    <row r="2708" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2708" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2708" s="18"/>
       <c r="C2708" s="1"/>
       <c r="D2708" s="1"/>
@@ -87704,7 +87703,7 @@
       <c r="G2708" s="10"/>
       <c r="K2708" s="7"/>
     </row>
-    <row r="2709" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2709" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2709" s="18"/>
       <c r="C2709" s="1"/>
       <c r="D2709" s="1"/>
@@ -87716,7 +87715,7 @@
       <c r="G2709" s="10"/>
       <c r="K2709" s="7"/>
     </row>
-    <row r="2710" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2710" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2710" s="18"/>
       <c r="C2710" s="1"/>
       <c r="D2710" s="1"/>
@@ -87728,7 +87727,7 @@
       <c r="G2710" s="10"/>
       <c r="K2710" s="7"/>
     </row>
-    <row r="2711" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2711" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2711" s="18"/>
       <c r="C2711" s="1"/>
       <c r="D2711" s="1"/>
@@ -87740,7 +87739,7 @@
       <c r="G2711" s="10"/>
       <c r="K2711" s="7"/>
     </row>
-    <row r="2712" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2712" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2712" s="18"/>
       <c r="C2712" s="1"/>
       <c r="D2712" s="1"/>
@@ -87752,7 +87751,7 @@
       <c r="G2712" s="10"/>
       <c r="K2712" s="7"/>
     </row>
-    <row r="2713" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2713" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2713" s="18"/>
       <c r="C2713" s="1"/>
       <c r="D2713" s="1"/>
@@ -87764,7 +87763,7 @@
       <c r="G2713" s="10"/>
       <c r="K2713" s="7"/>
     </row>
-    <row r="2714" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2714" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2714" s="18"/>
       <c r="C2714" s="1"/>
       <c r="D2714" s="1"/>
@@ -87776,7 +87775,7 @@
       <c r="G2714" s="10"/>
       <c r="K2714" s="7"/>
     </row>
-    <row r="2715" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2715" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2715" s="18"/>
       <c r="C2715" s="1"/>
       <c r="D2715" s="1"/>
@@ -87788,7 +87787,7 @@
       <c r="G2715" s="10"/>
       <c r="K2715" s="7"/>
     </row>
-    <row r="2716" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2716" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2716" s="18"/>
       <c r="C2716" s="1"/>
       <c r="D2716" s="1"/>
@@ -87800,7 +87799,7 @@
       <c r="G2716" s="10"/>
       <c r="K2716" s="7"/>
     </row>
-    <row r="2717" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2717" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2717" s="18"/>
       <c r="C2717" s="1"/>
       <c r="D2717" s="1"/>
@@ -87812,7 +87811,7 @@
       <c r="G2717" s="10"/>
       <c r="K2717" s="7"/>
     </row>
-    <row r="2718" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2718" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2718" s="18"/>
       <c r="C2718" s="1"/>
       <c r="D2718" s="1"/>
@@ -87824,7 +87823,7 @@
       <c r="G2718" s="10"/>
       <c r="K2718" s="7"/>
     </row>
-    <row r="2719" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2719" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2719" s="18"/>
       <c r="C2719" s="1"/>
       <c r="D2719" s="1"/>
@@ -87836,7 +87835,7 @@
       <c r="G2719" s="10"/>
       <c r="K2719" s="7"/>
     </row>
-    <row r="2720" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2720" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2720" s="18"/>
       <c r="C2720" s="1"/>
       <c r="D2720" s="1"/>
@@ -87848,7 +87847,7 @@
       <c r="G2720" s="10"/>
       <c r="K2720" s="7"/>
     </row>
-    <row r="2721" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2721" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2721" s="18"/>
       <c r="C2721" s="1"/>
       <c r="D2721" s="1"/>
@@ -87860,7 +87859,7 @@
       <c r="G2721" s="10"/>
       <c r="K2721" s="7"/>
     </row>
-    <row r="2722" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2722" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2722" s="18"/>
       <c r="C2722" s="1"/>
       <c r="D2722" s="1"/>
@@ -87872,7 +87871,7 @@
       <c r="G2722" s="10"/>
       <c r="K2722" s="7"/>
     </row>
-    <row r="2723" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2723" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2723" s="18"/>
       <c r="C2723" s="1"/>
       <c r="D2723" s="1"/>
@@ -87884,7 +87883,7 @@
       <c r="G2723" s="10"/>
       <c r="K2723" s="7"/>
     </row>
-    <row r="2724" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2724" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2724" s="18"/>
       <c r="C2724" s="1"/>
       <c r="D2724" s="1"/>
@@ -87896,7 +87895,7 @@
       <c r="G2724" s="10"/>
       <c r="K2724" s="7"/>
     </row>
-    <row r="2725" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2725" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2725" s="18"/>
       <c r="C2725" s="1"/>
       <c r="D2725" s="1"/>
@@ -87908,7 +87907,7 @@
       <c r="G2725" s="10"/>
       <c r="K2725" s="7"/>
     </row>
-    <row r="2726" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2726" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2726" s="18"/>
       <c r="C2726" s="1"/>
       <c r="D2726" s="1"/>
@@ -87920,7 +87919,7 @@
       <c r="G2726" s="10"/>
       <c r="K2726" s="7"/>
     </row>
-    <row r="2727" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2727" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2727" s="18"/>
       <c r="C2727" s="1"/>
       <c r="D2727" s="1"/>
@@ -87932,7 +87931,7 @@
       <c r="G2727" s="10"/>
       <c r="K2727" s="7"/>
     </row>
-    <row r="2728" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2728" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2728" s="18"/>
       <c r="C2728" s="1"/>
       <c r="D2728" s="1"/>
@@ -87944,7 +87943,7 @@
       <c r="G2728" s="10"/>
       <c r="K2728" s="7"/>
     </row>
-    <row r="2729" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2729" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2729" s="18"/>
       <c r="C2729" s="1"/>
       <c r="D2729" s="1"/>
@@ -87956,7 +87955,7 @@
       <c r="G2729" s="10"/>
       <c r="K2729" s="7"/>
     </row>
-    <row r="2730" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2730" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2730" s="18"/>
       <c r="C2730" s="1"/>
       <c r="D2730" s="1"/>
@@ -87968,7 +87967,7 @@
       <c r="G2730" s="10"/>
       <c r="K2730" s="7"/>
     </row>
-    <row r="2731" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2731" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2731" s="18"/>
       <c r="C2731" s="1"/>
       <c r="D2731" s="1"/>
@@ -87980,7 +87979,7 @@
       <c r="G2731" s="10"/>
       <c r="K2731" s="7"/>
     </row>
-    <row r="2732" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2732" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2732" s="18"/>
       <c r="C2732" s="1"/>
       <c r="D2732" s="1"/>
@@ -87992,7 +87991,7 @@
       <c r="G2732" s="10"/>
       <c r="K2732" s="7"/>
     </row>
-    <row r="2733" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2733" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2733" s="18"/>
       <c r="C2733" s="1"/>
       <c r="D2733" s="1"/>
@@ -88004,7 +88003,7 @@
       <c r="G2733" s="10"/>
       <c r="K2733" s="7"/>
     </row>
-    <row r="2734" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2734" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2734" s="18"/>
       <c r="C2734" s="1"/>
       <c r="D2734" s="1"/>
@@ -88016,7 +88015,7 @@
       <c r="G2734" s="10"/>
       <c r="K2734" s="7"/>
     </row>
-    <row r="2735" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2735" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2735" s="18"/>
       <c r="C2735" s="1"/>
       <c r="D2735" s="1"/>
@@ -88028,7 +88027,7 @@
       <c r="G2735" s="10"/>
       <c r="K2735" s="7"/>
     </row>
-    <row r="2736" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2736" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2736" s="18"/>
       <c r="C2736" s="1"/>
       <c r="D2736" s="1"/>
@@ -88040,7 +88039,7 @@
       <c r="G2736" s="10"/>
       <c r="K2736" s="7"/>
     </row>
-    <row r="2737" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2737" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2737" s="18"/>
       <c r="C2737" s="1"/>
       <c r="D2737" s="1"/>
@@ -88052,7 +88051,7 @@
       <c r="G2737" s="10"/>
       <c r="K2737" s="7"/>
     </row>
-    <row r="2738" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2738" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2738" s="18"/>
       <c r="C2738" s="1"/>
       <c r="D2738" s="1"/>
@@ -88064,7 +88063,7 @@
       <c r="G2738" s="10"/>
       <c r="K2738" s="7"/>
     </row>
-    <row r="2739" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2739" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2739" s="18"/>
       <c r="C2739" s="1"/>
       <c r="D2739" s="1"/>
@@ -88076,7 +88075,7 @@
       <c r="G2739" s="10"/>
       <c r="K2739" s="7"/>
     </row>
-    <row r="2740" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2740" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2740" s="18"/>
       <c r="C2740" s="1"/>
       <c r="D2740" s="1"/>
@@ -88088,7 +88087,7 @@
       <c r="G2740" s="10"/>
       <c r="K2740" s="7"/>
     </row>
-    <row r="2741" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2741" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2741" s="18"/>
       <c r="C2741" s="1"/>
       <c r="D2741" s="1"/>
@@ -88100,7 +88099,7 @@
       <c r="G2741" s="10"/>
       <c r="K2741" s="7"/>
     </row>
-    <row r="2742" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2742" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2742" s="18"/>
       <c r="C2742" s="1"/>
       <c r="D2742" s="1"/>
@@ -88112,7 +88111,7 @@
       <c r="G2742" s="10"/>
       <c r="K2742" s="7"/>
     </row>
-    <row r="2743" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2743" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2743" s="18"/>
       <c r="C2743" s="1"/>
       <c r="D2743" s="1"/>
@@ -88124,7 +88123,7 @@
       <c r="G2743" s="10"/>
       <c r="K2743" s="7"/>
     </row>
-    <row r="2744" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2744" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2744" s="18"/>
       <c r="C2744" s="1"/>
       <c r="D2744" s="1"/>
@@ -88136,7 +88135,7 @@
       <c r="G2744" s="10"/>
       <c r="K2744" s="7"/>
     </row>
-    <row r="2745" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2745" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2745" s="18"/>
       <c r="C2745" s="1"/>
       <c r="D2745" s="1"/>
@@ -88148,7 +88147,7 @@
       <c r="G2745" s="10"/>
       <c r="K2745" s="7"/>
     </row>
-    <row r="2746" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2746" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2746" s="18"/>
       <c r="C2746" s="1"/>
       <c r="D2746" s="1"/>
@@ -88160,7 +88159,7 @@
       <c r="G2746" s="10"/>
       <c r="K2746" s="7"/>
     </row>
-    <row r="2747" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2747" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2747" s="18"/>
       <c r="C2747" s="1"/>
       <c r="D2747" s="1"/>
@@ -88172,7 +88171,7 @@
       <c r="G2747" s="10"/>
       <c r="K2747" s="7"/>
     </row>
-    <row r="2748" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2748" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2748" s="18"/>
       <c r="C2748" s="1"/>
       <c r="D2748" s="1"/>
@@ -88184,7 +88183,7 @@
       <c r="G2748" s="10"/>
       <c r="K2748" s="7"/>
     </row>
-    <row r="2749" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2749" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2749" s="18"/>
       <c r="C2749" s="1"/>
       <c r="D2749" s="1"/>
@@ -88196,7 +88195,7 @@
       <c r="G2749" s="10"/>
       <c r="K2749" s="7"/>
     </row>
-    <row r="2750" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2750" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2750" s="18"/>
       <c r="C2750" s="1"/>
       <c r="D2750" s="1"/>
@@ -88208,7 +88207,7 @@
       <c r="G2750" s="10"/>
       <c r="K2750" s="7"/>
     </row>
-    <row r="2751" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2751" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2751" s="18"/>
       <c r="C2751" s="1"/>
       <c r="D2751" s="1"/>
@@ -88220,7 +88219,7 @@
       <c r="G2751" s="10"/>
       <c r="K2751" s="7"/>
     </row>
-    <row r="2752" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2752" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2752" s="18"/>
       <c r="C2752" s="1"/>
       <c r="D2752" s="1"/>
@@ -88232,7 +88231,7 @@
       <c r="G2752" s="10"/>
       <c r="K2752" s="7"/>
     </row>
-    <row r="2753" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2753" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2753" s="18"/>
       <c r="C2753" s="1"/>
       <c r="D2753" s="1"/>
@@ -88244,7 +88243,7 @@
       <c r="G2753" s="10"/>
       <c r="K2753" s="7"/>
     </row>
-    <row r="2754" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2754" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2754" s="18"/>
       <c r="C2754" s="1"/>
       <c r="D2754" s="1"/>
@@ -88256,7 +88255,7 @@
       <c r="G2754" s="10"/>
       <c r="K2754" s="7"/>
     </row>
-    <row r="2755" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2755" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2755" s="18"/>
       <c r="C2755" s="1"/>
       <c r="D2755" s="1"/>
@@ -88268,7 +88267,7 @@
       <c r="G2755" s="10"/>
       <c r="K2755" s="7"/>
     </row>
-    <row r="2756" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2756" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2756" s="18"/>
       <c r="C2756" s="1"/>
       <c r="D2756" s="1"/>
@@ -88280,7 +88279,7 @@
       <c r="G2756" s="10"/>
       <c r="K2756" s="7"/>
     </row>
-    <row r="2757" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2757" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2757" s="18"/>
       <c r="C2757" s="1"/>
       <c r="D2757" s="1"/>
@@ -88292,7 +88291,7 @@
       <c r="G2757" s="10"/>
       <c r="K2757" s="7"/>
     </row>
-    <row r="2758" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2758" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2758" s="18"/>
       <c r="C2758" s="1"/>
       <c r="D2758" s="1"/>
@@ -88304,7 +88303,7 @@
       <c r="G2758" s="10"/>
       <c r="K2758" s="7"/>
     </row>
-    <row r="2759" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2759" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2759" s="18"/>
       <c r="C2759" s="1"/>
       <c r="D2759" s="1"/>
@@ -88316,7 +88315,7 @@
       <c r="G2759" s="10"/>
       <c r="K2759" s="7"/>
     </row>
-    <row r="2760" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2760" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2760" s="18"/>
       <c r="C2760" s="1"/>
       <c r="D2760" s="1"/>
@@ -88328,7 +88327,7 @@
       <c r="G2760" s="10"/>
       <c r="K2760" s="7"/>
     </row>
-    <row r="2761" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2761" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2761" s="18"/>
       <c r="C2761" s="1"/>
       <c r="D2761" s="1"/>
@@ -88340,7 +88339,7 @@
       <c r="G2761" s="10"/>
       <c r="K2761" s="7"/>
     </row>
-    <row r="2762" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2762" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2762" s="18"/>
       <c r="C2762" s="1"/>
       <c r="D2762" s="1"/>
@@ -88352,7 +88351,7 @@
       <c r="G2762" s="10"/>
       <c r="K2762" s="7"/>
     </row>
-    <row r="2763" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2763" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2763" s="18"/>
       <c r="C2763" s="1"/>
       <c r="D2763" s="1"/>
@@ -88364,7 +88363,7 @@
       <c r="G2763" s="10"/>
       <c r="K2763" s="7"/>
     </row>
-    <row r="2764" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2764" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2764" s="18"/>
       <c r="C2764" s="1"/>
       <c r="D2764" s="1"/>
@@ -88376,7 +88375,7 @@
       <c r="G2764" s="10"/>
       <c r="K2764" s="7"/>
     </row>
-    <row r="2765" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2765" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2765" s="18"/>
       <c r="C2765" s="1"/>
       <c r="D2765" s="1"/>
@@ -88388,7 +88387,7 @@
       <c r="G2765" s="10"/>
       <c r="K2765" s="7"/>
     </row>
-    <row r="2766" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2766" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2766" s="18"/>
       <c r="C2766" s="1"/>
       <c r="D2766" s="1"/>
@@ -88400,7 +88399,7 @@
       <c r="G2766" s="10"/>
       <c r="K2766" s="7"/>
     </row>
-    <row r="2767" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2767" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2767" s="18"/>
       <c r="C2767" s="1"/>
       <c r="D2767" s="1"/>
@@ -88412,7 +88411,7 @@
       <c r="G2767" s="10"/>
       <c r="K2767" s="7"/>
     </row>
-    <row r="2768" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2768" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2768" s="18"/>
       <c r="C2768" s="1"/>
       <c r="D2768" s="1"/>
@@ -88424,7 +88423,7 @@
       <c r="G2768" s="10"/>
       <c r="K2768" s="7"/>
     </row>
-    <row r="2769" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2769" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2769" s="18"/>
       <c r="C2769" s="1"/>
       <c r="D2769" s="1"/>
@@ -88436,7 +88435,7 @@
       <c r="G2769" s="10"/>
       <c r="K2769" s="7"/>
     </row>
-    <row r="2770" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2770" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2770" s="18"/>
       <c r="C2770" s="1"/>
       <c r="D2770" s="1"/>
@@ -88448,7 +88447,7 @@
       <c r="G2770" s="10"/>
       <c r="K2770" s="7"/>
     </row>
-    <row r="2771" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2771" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2771" s="18"/>
       <c r="C2771" s="1"/>
       <c r="D2771" s="1"/>
@@ -88460,7 +88459,7 @@
       <c r="G2771" s="10"/>
       <c r="K2771" s="7"/>
     </row>
-    <row r="2772" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2772" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2772" s="18"/>
       <c r="C2772" s="1"/>
       <c r="D2772" s="1"/>
@@ -88472,7 +88471,7 @@
       <c r="G2772" s="10"/>
       <c r="K2772" s="7"/>
     </row>
-    <row r="2773" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2773" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2773" s="18"/>
       <c r="C2773" s="1"/>
       <c r="D2773" s="1"/>
@@ -88484,7 +88483,7 @@
       <c r="G2773" s="10"/>
       <c r="K2773" s="7"/>
     </row>
-    <row r="2774" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2774" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2774" s="18"/>
       <c r="C2774" s="1"/>
       <c r="D2774" s="1"/>
@@ -88496,7 +88495,7 @@
       <c r="G2774" s="10"/>
       <c r="K2774" s="7"/>
     </row>
-    <row r="2775" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2775" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2775" s="18"/>
       <c r="C2775" s="1"/>
       <c r="D2775" s="1"/>
@@ -88508,7 +88507,7 @@
       <c r="G2775" s="10"/>
       <c r="K2775" s="7"/>
     </row>
-    <row r="2776" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2776" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2776" s="18"/>
       <c r="C2776" s="1"/>
       <c r="D2776" s="1"/>
@@ -88520,7 +88519,7 @@
       <c r="G2776" s="10"/>
       <c r="K2776" s="7"/>
     </row>
-    <row r="2777" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2777" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2777" s="18"/>
       <c r="C2777" s="1"/>
       <c r="D2777" s="1"/>
@@ -88532,7 +88531,7 @@
       <c r="G2777" s="10"/>
       <c r="K2777" s="7"/>
     </row>
-    <row r="2778" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2778" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2778" s="18"/>
       <c r="C2778" s="1"/>
       <c r="D2778" s="1"/>
@@ -88544,7 +88543,7 @@
       <c r="G2778" s="10"/>
       <c r="K2778" s="7"/>
     </row>
-    <row r="2779" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2779" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2779" s="18"/>
       <c r="C2779" s="1"/>
       <c r="D2779" s="1"/>
@@ -88556,7 +88555,7 @@
       <c r="G2779" s="10"/>
       <c r="K2779" s="7"/>
     </row>
-    <row r="2780" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2780" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2780" s="18"/>
       <c r="C2780" s="1"/>
       <c r="D2780" s="1"/>
@@ -88568,7 +88567,7 @@
       <c r="G2780" s="10"/>
       <c r="K2780" s="7"/>
     </row>
-    <row r="2781" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2781" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2781" s="18"/>
       <c r="C2781" s="1"/>
       <c r="D2781" s="1"/>
@@ -88580,7 +88579,7 @@
       <c r="G2781" s="10"/>
       <c r="K2781" s="7"/>
     </row>
-    <row r="2782" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2782" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2782" s="18"/>
       <c r="C2782" s="1"/>
       <c r="D2782" s="1"/>
@@ -88592,7 +88591,7 @@
       <c r="G2782" s="10"/>
       <c r="K2782" s="7"/>
     </row>
-    <row r="2783" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2783" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2783" s="18"/>
       <c r="C2783" s="1"/>
       <c r="D2783" s="1"/>
@@ -88604,7 +88603,7 @@
       <c r="G2783" s="10"/>
       <c r="K2783" s="7"/>
     </row>
-    <row r="2784" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2784" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2784" s="18"/>
       <c r="C2784" s="1"/>
       <c r="D2784" s="1"/>
@@ -88616,7 +88615,7 @@
       <c r="G2784" s="10"/>
       <c r="K2784" s="7"/>
     </row>
-    <row r="2785" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2785" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2785" s="18"/>
       <c r="C2785" s="1"/>
       <c r="D2785" s="1"/>
@@ -88628,7 +88627,7 @@
       <c r="G2785" s="10"/>
       <c r="K2785" s="7"/>
     </row>
-    <row r="2786" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2786" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2786" s="18"/>
       <c r="C2786" s="1"/>
       <c r="D2786" s="1"/>
@@ -88640,7 +88639,7 @@
       <c r="G2786" s="10"/>
       <c r="K2786" s="7"/>
     </row>
-    <row r="2787" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2787" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2787" s="18"/>
       <c r="C2787" s="1"/>
       <c r="D2787" s="1"/>
@@ -88652,7 +88651,7 @@
       <c r="G2787" s="10"/>
       <c r="K2787" s="7"/>
     </row>
-    <row r="2788" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2788" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2788" s="18"/>
       <c r="C2788" s="1"/>
       <c r="D2788" s="1"/>
@@ -88664,7 +88663,7 @@
       <c r="G2788" s="10"/>
       <c r="K2788" s="7"/>
     </row>
-    <row r="2789" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2789" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2789" s="18"/>
       <c r="C2789" s="1"/>
       <c r="D2789" s="1"/>
@@ -88676,7 +88675,7 @@
       <c r="G2789" s="10"/>
       <c r="K2789" s="7"/>
     </row>
-    <row r="2790" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2790" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2790" s="18"/>
       <c r="C2790" s="1"/>
       <c r="D2790" s="1"/>
@@ -88688,7 +88687,7 @@
       <c r="G2790" s="10"/>
       <c r="K2790" s="7"/>
     </row>
-    <row r="2791" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2791" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2791" s="18"/>
       <c r="C2791" s="1"/>
       <c r="D2791" s="1"/>
@@ -88700,7 +88699,7 @@
       <c r="G2791" s="10"/>
       <c r="K2791" s="7"/>
     </row>
-    <row r="2792" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2792" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2792" s="18"/>
       <c r="C2792" s="1"/>
       <c r="D2792" s="1"/>
@@ -88712,7 +88711,7 @@
       <c r="G2792" s="10"/>
       <c r="K2792" s="7"/>
     </row>
-    <row r="2793" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2793" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2793" s="18"/>
       <c r="C2793" s="1"/>
       <c r="D2793" s="1"/>
@@ -88724,7 +88723,7 @@
       <c r="G2793" s="10"/>
       <c r="K2793" s="7"/>
     </row>
-    <row r="2794" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2794" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2794" s="18"/>
       <c r="C2794" s="1"/>
       <c r="D2794" s="1"/>
@@ -88736,7 +88735,7 @@
       <c r="G2794" s="10"/>
       <c r="K2794" s="7"/>
     </row>
-    <row r="2795" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2795" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2795" s="18"/>
       <c r="C2795" s="1"/>
       <c r="D2795" s="1"/>
@@ -88748,7 +88747,7 @@
       <c r="G2795" s="10"/>
       <c r="K2795" s="7"/>
     </row>
-    <row r="2796" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2796" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2796" s="18"/>
       <c r="C2796" s="1"/>
       <c r="D2796" s="1"/>
@@ -88760,7 +88759,7 @@
       <c r="G2796" s="10"/>
       <c r="K2796" s="7"/>
     </row>
-    <row r="2797" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2797" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2797" s="18"/>
       <c r="C2797" s="1"/>
       <c r="D2797" s="1"/>
@@ -88772,7 +88771,7 @@
       <c r="G2797" s="10"/>
       <c r="K2797" s="7"/>
     </row>
-    <row r="2798" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2798" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2798" s="18"/>
       <c r="C2798" s="1"/>
       <c r="D2798" s="1"/>
@@ -88784,7 +88783,7 @@
       <c r="G2798" s="10"/>
       <c r="K2798" s="7"/>
     </row>
-    <row r="2799" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2799" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2799" s="18"/>
       <c r="C2799" s="1"/>
       <c r="D2799" s="1"/>
@@ -88796,7 +88795,7 @@
       <c r="G2799" s="10"/>
       <c r="K2799" s="7"/>
     </row>
-    <row r="2800" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2800" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2800" s="18"/>
       <c r="C2800" s="1"/>
       <c r="D2800" s="1"/>
@@ -88808,7 +88807,7 @@
       <c r="G2800" s="10"/>
       <c r="K2800" s="7"/>
     </row>
-    <row r="2801" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2801" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2801" s="18"/>
       <c r="C2801" s="1"/>
       <c r="D2801" s="1"/>
@@ -88820,7 +88819,7 @@
       <c r="G2801" s="10"/>
       <c r="K2801" s="7"/>
     </row>
-    <row r="2802" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2802" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2802" s="18"/>
       <c r="C2802" s="1"/>
       <c r="D2802" s="1"/>
@@ -88832,7 +88831,7 @@
       <c r="G2802" s="10"/>
       <c r="K2802" s="7"/>
     </row>
-    <row r="2803" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2803" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2803" s="18"/>
       <c r="C2803" s="1"/>
       <c r="D2803" s="1"/>
@@ -88844,7 +88843,7 @@
       <c r="G2803" s="10"/>
       <c r="K2803" s="7"/>
     </row>
-    <row r="2804" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2804" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2804" s="18"/>
       <c r="C2804" s="1"/>
       <c r="D2804" s="1"/>
@@ -88856,7 +88855,7 @@
       <c r="G2804" s="10"/>
       <c r="K2804" s="7"/>
     </row>
-    <row r="2805" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2805" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2805" s="18"/>
       <c r="C2805" s="1"/>
       <c r="D2805" s="1"/>
@@ -88868,7 +88867,7 @@
       <c r="G2805" s="10"/>
       <c r="K2805" s="7"/>
     </row>
-    <row r="2806" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2806" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2806" s="18"/>
       <c r="C2806" s="1"/>
       <c r="D2806" s="1"/>
@@ -88880,7 +88879,7 @@
       <c r="G2806" s="10"/>
       <c r="K2806" s="7"/>
     </row>
-    <row r="2807" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2807" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2807" s="18"/>
       <c r="C2807" s="1"/>
       <c r="D2807" s="1"/>
@@ -88892,7 +88891,7 @@
       <c r="G2807" s="10"/>
       <c r="K2807" s="7"/>
     </row>
-    <row r="2808" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2808" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2808" s="18"/>
       <c r="C2808" s="1"/>
       <c r="D2808" s="1"/>
@@ -88904,7 +88903,7 @@
       <c r="G2808" s="10"/>
       <c r="K2808" s="7"/>
     </row>
-    <row r="2809" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2809" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2809" s="18"/>
       <c r="C2809" s="1"/>
       <c r="D2809" s="1"/>
@@ -88916,7 +88915,7 @@
       <c r="G2809" s="10"/>
       <c r="K2809" s="7"/>
     </row>
-    <row r="2810" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2810" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2810" s="18"/>
       <c r="C2810" s="1"/>
       <c r="D2810" s="1"/>
@@ -88928,7 +88927,7 @@
       <c r="G2810" s="10"/>
       <c r="K2810" s="7"/>
     </row>
-    <row r="2811" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2811" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2811" s="18"/>
       <c r="C2811" s="1"/>
       <c r="D2811" s="1"/>
@@ -88940,7 +88939,7 @@
       <c r="G2811" s="10"/>
       <c r="K2811" s="7"/>
     </row>
-    <row r="2812" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2812" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2812" s="18"/>
       <c r="C2812" s="1"/>
       <c r="D2812" s="1"/>
@@ -88952,7 +88951,7 @@
       <c r="G2812" s="10"/>
       <c r="K2812" s="7"/>
     </row>
-    <row r="2813" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2813" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2813" s="18"/>
       <c r="C2813" s="1"/>
       <c r="D2813" s="1"/>
@@ -88964,7 +88963,7 @@
       <c r="G2813" s="10"/>
       <c r="K2813" s="7"/>
     </row>
-    <row r="2814" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2814" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2814" s="18"/>
       <c r="C2814" s="1"/>
       <c r="D2814" s="1"/>
@@ -88976,7 +88975,7 @@
       <c r="G2814" s="10"/>
       <c r="K2814" s="7"/>
     </row>
-    <row r="2815" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2815" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2815" s="18"/>
       <c r="C2815" s="1"/>
       <c r="D2815" s="1"/>
@@ -88988,7 +88987,7 @@
       <c r="G2815" s="10"/>
       <c r="K2815" s="7"/>
     </row>
-    <row r="2816" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2816" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2816" s="18"/>
       <c r="C2816" s="1"/>
       <c r="D2816" s="1"/>
@@ -89000,7 +88999,7 @@
       <c r="G2816" s="10"/>
       <c r="K2816" s="7"/>
     </row>
-    <row r="2817" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2817" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2817" s="18"/>
       <c r="C2817" s="1"/>
       <c r="D2817" s="1"/>
@@ -89012,7 +89011,7 @@
       <c r="G2817" s="10"/>
       <c r="K2817" s="7"/>
     </row>
-    <row r="2818" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2818" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2818" s="18"/>
       <c r="C2818" s="1"/>
       <c r="D2818" s="1"/>
@@ -89024,7 +89023,7 @@
       <c r="G2818" s="10"/>
       <c r="K2818" s="7"/>
     </row>
-    <row r="2819" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2819" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2819" s="18"/>
       <c r="C2819" s="1"/>
       <c r="D2819" s="1"/>
@@ -89036,7 +89035,7 @@
       <c r="G2819" s="10"/>
       <c r="K2819" s="7"/>
     </row>
-    <row r="2820" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2820" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2820" s="18"/>
       <c r="C2820" s="1"/>
       <c r="D2820" s="1"/>
@@ -89048,7 +89047,7 @@
       <c r="G2820" s="10"/>
       <c r="K2820" s="7"/>
     </row>
-    <row r="2821" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2821" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2821" s="18"/>
       <c r="C2821" s="1"/>
       <c r="D2821" s="1"/>
@@ -89060,7 +89059,7 @@
       <c r="G2821" s="10"/>
       <c r="K2821" s="7"/>
     </row>
-    <row r="2822" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2822" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2822" s="18"/>
       <c r="C2822" s="1"/>
       <c r="D2822" s="1"/>
@@ -89072,7 +89071,7 @@
       <c r="G2822" s="10"/>
       <c r="K2822" s="7"/>
     </row>
-    <row r="2823" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2823" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2823" s="18"/>
       <c r="C2823" s="1"/>
       <c r="D2823" s="1"/>
@@ -89084,7 +89083,7 @@
       <c r="G2823" s="10"/>
       <c r="K2823" s="7"/>
     </row>
-    <row r="2824" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2824" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2824" s="18"/>
       <c r="C2824" s="1"/>
       <c r="D2824" s="1"/>
@@ -89096,7 +89095,7 @@
       <c r="G2824" s="10"/>
       <c r="K2824" s="7"/>
     </row>
-    <row r="2825" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2825" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2825" s="18"/>
       <c r="C2825" s="1"/>
       <c r="D2825" s="1"/>
@@ -89108,7 +89107,7 @@
       <c r="G2825" s="10"/>
       <c r="K2825" s="7"/>
     </row>
-    <row r="2826" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2826" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2826" s="18"/>
       <c r="C2826" s="1"/>
       <c r="D2826" s="1"/>
@@ -89120,7 +89119,7 @@
       <c r="G2826" s="10"/>
       <c r="K2826" s="7"/>
     </row>
-    <row r="2827" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2827" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2827" s="18"/>
       <c r="C2827" s="1"/>
       <c r="D2827" s="1"/>
@@ -89132,7 +89131,7 @@
       <c r="G2827" s="10"/>
       <c r="K2827" s="7"/>
     </row>
-    <row r="2828" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2828" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2828" s="18"/>
       <c r="C2828" s="1"/>
       <c r="D2828" s="1"/>
@@ -89144,7 +89143,7 @@
       <c r="G2828" s="10"/>
       <c r="K2828" s="7"/>
     </row>
-    <row r="2829" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2829" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2829" s="18"/>
       <c r="C2829" s="1"/>
       <c r="D2829" s="1"/>
@@ -89156,7 +89155,7 @@
       <c r="G2829" s="10"/>
       <c r="K2829" s="7"/>
     </row>
-    <row r="2830" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2830" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2830" s="18"/>
       <c r="C2830" s="1"/>
       <c r="D2830" s="1"/>
@@ -89168,7 +89167,7 @@
       <c r="G2830" s="10"/>
       <c r="K2830" s="7"/>
     </row>
-    <row r="2831" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2831" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2831" s="18"/>
       <c r="C2831" s="1"/>
       <c r="D2831" s="1"/>
@@ -89180,7 +89179,7 @@
       <c r="G2831" s="10"/>
       <c r="K2831" s="7"/>
     </row>
-    <row r="2832" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2832" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2832" s="18"/>
       <c r="C2832" s="1"/>
       <c r="D2832" s="1"/>
@@ -89192,7 +89191,7 @@
       <c r="G2832" s="10"/>
       <c r="K2832" s="7"/>
     </row>
-    <row r="2833" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2833" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2833" s="18"/>
       <c r="C2833" s="1"/>
       <c r="D2833" s="1"/>
@@ -89204,7 +89203,7 @@
       <c r="G2833" s="10"/>
       <c r="K2833" s="7"/>
     </row>
-    <row r="2834" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2834" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2834" s="18"/>
       <c r="C2834" s="1"/>
       <c r="D2834" s="1"/>
@@ -89216,7 +89215,7 @@
       <c r="G2834" s="10"/>
       <c r="K2834" s="7"/>
     </row>
-    <row r="2835" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2835" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2835" s="18"/>
       <c r="C2835" s="1"/>
       <c r="D2835" s="1"/>
@@ -89228,7 +89227,7 @@
       <c r="G2835" s="10"/>
       <c r="K2835" s="7"/>
     </row>
-    <row r="2836" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2836" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2836" s="18"/>
       <c r="C2836" s="1"/>
       <c r="D2836" s="1"/>
@@ -89240,7 +89239,7 @@
       <c r="G2836" s="10"/>
       <c r="K2836" s="7"/>
     </row>
-    <row r="2837" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2837" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2837" s="18"/>
       <c r="C2837" s="1"/>
       <c r="D2837" s="1"/>
@@ -89252,7 +89251,7 @@
       <c r="G2837" s="10"/>
       <c r="K2837" s="7"/>
     </row>
-    <row r="2838" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2838" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2838" s="18"/>
       <c r="C2838" s="1"/>
       <c r="D2838" s="1"/>
@@ -89264,7 +89263,7 @@
       <c r="G2838" s="10"/>
       <c r="K2838" s="7"/>
     </row>
-    <row r="2839" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2839" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2839" s="18"/>
       <c r="C2839" s="1"/>
       <c r="D2839" s="1"/>
@@ -89276,7 +89275,7 @@
       <c r="G2839" s="10"/>
       <c r="K2839" s="7"/>
     </row>
-    <row r="2840" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2840" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2840" s="18"/>
       <c r="C2840" s="1"/>
       <c r="D2840" s="1"/>
@@ -89288,7 +89287,7 @@
       <c r="G2840" s="10"/>
       <c r="K2840" s="7"/>
     </row>
-    <row r="2841" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2841" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2841" s="18"/>
       <c r="C2841" s="1"/>
       <c r="D2841" s="1"/>
@@ -89300,7 +89299,7 @@
       <c r="G2841" s="10"/>
       <c r="K2841" s="7"/>
     </row>
-    <row r="2842" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2842" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2842" s="18"/>
       <c r="C2842" s="1"/>
       <c r="D2842" s="1"/>
@@ -89312,7 +89311,7 @@
       <c r="G2842" s="10"/>
       <c r="K2842" s="7"/>
     </row>
-    <row r="2843" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2843" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2843" s="18"/>
       <c r="C2843" s="1"/>
       <c r="D2843" s="1"/>
@@ -89324,7 +89323,7 @@
       <c r="G2843" s="10"/>
       <c r="K2843" s="7"/>
     </row>
-    <row r="2844" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2844" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2844" s="18"/>
       <c r="C2844" s="1"/>
       <c r="D2844" s="1"/>
@@ -89336,7 +89335,7 @@
       <c r="G2844" s="10"/>
       <c r="K2844" s="7"/>
     </row>
-    <row r="2845" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2845" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2845" s="18"/>
       <c r="C2845" s="1"/>
       <c r="D2845" s="1"/>
@@ -89348,7 +89347,7 @@
       <c r="G2845" s="10"/>
       <c r="K2845" s="7"/>
     </row>
-    <row r="2846" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2846" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2846" s="18"/>
       <c r="C2846" s="1"/>
       <c r="D2846" s="1"/>
@@ -89360,7 +89359,7 @@
       <c r="G2846" s="10"/>
       <c r="K2846" s="7"/>
     </row>
-    <row r="2847" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2847" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2847" s="18"/>
       <c r="C2847" s="1"/>
       <c r="D2847" s="1"/>
@@ -89372,7 +89371,7 @@
       <c r="G2847" s="10"/>
       <c r="K2847" s="7"/>
     </row>
-    <row r="2848" spans="2:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2848" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2848" s="18"/>
       <c r="C2848" s="1"/>
       <c r="D2848" s="1"/>
@@ -89454,13 +89453,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B2:L2851" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-    <filterColumn colId="7">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B2:L2851" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-21 12:49
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="990" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F7E4FB6-AD86-4141-A6D9-9D62AAB87473}"/>
+  <xr:revisionPtr revIDLastSave="1169" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11AD6616-EAAF-49F5-B597-951874DF896B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8230" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8298" uniqueCount="340">
   <si>
     <t>Data</t>
   </si>
@@ -1054,6 +1054,12 @@
   <si>
     <t>PAREBEM POSTO NITEROI</t>
   </si>
+  <si>
+    <t>HJF5G06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REDE DOM PEDRO DE POSTOS </t>
+  </si>
 </sst>
 </file>
 
@@ -87037,24 +87043,541 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2659" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="2653" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2653" s="23">
+        <v>45945</v>
+      </c>
+      <c r="F2653" s="2">
+        <v>56.716000000000001</v>
+      </c>
+      <c r="G2653" s="2">
+        <v>347.1</v>
+      </c>
+      <c r="H2653" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2653" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2653" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2653" s="2" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="2654" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2654" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2654" s="2">
+        <v>134.29</v>
+      </c>
+      <c r="G2654" s="2">
+        <v>858.11</v>
+      </c>
+      <c r="H2654" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2654" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2654" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="K2654" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2655" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2655" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2655" s="2">
+        <v>100.94</v>
+      </c>
+      <c r="G2655" s="2">
+        <v>593.53</v>
+      </c>
+      <c r="H2655" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2655" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2655" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2655" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2656" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2656" s="23">
+        <v>45948</v>
+      </c>
+      <c r="F2656" s="2">
+        <v>99.33</v>
+      </c>
+      <c r="G2656" s="2">
+        <v>600</v>
+      </c>
+      <c r="H2656" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2656" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2656" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2656" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2657" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2657" s="23">
+        <v>45945</v>
+      </c>
+      <c r="F2657" s="2">
+        <v>201.63</v>
+      </c>
+      <c r="G2657" s="2">
+        <v>1268.26</v>
+      </c>
+      <c r="H2657" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2657" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2657" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2657" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2658" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2658" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2658" s="2">
+        <v>231.483</v>
+      </c>
+      <c r="G2658" s="2">
+        <v>1361.12</v>
+      </c>
+      <c r="H2658" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2658" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2658" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2658" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2659" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2659" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2659" s="2">
+        <v>126.08199999999999</v>
+      </c>
+      <c r="G2659" s="2">
+        <v>741.36</v>
+      </c>
+      <c r="H2659" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2659" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2659" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2659" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="L2659" s="28"/>
     </row>
-    <row r="2670" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="2660" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2660" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2660" s="2">
+        <v>170.85</v>
+      </c>
+      <c r="G2660" s="2">
+        <v>1108.82</v>
+      </c>
+      <c r="H2660" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2660" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2660" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2660" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2661" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2661" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2661" s="2">
+        <v>85.617999999999995</v>
+      </c>
+      <c r="G2661" s="2">
+        <v>500</v>
+      </c>
+      <c r="H2661" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2661" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2661" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="K2661" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2662" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2662" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2662" s="2">
+        <v>146.61099999999999</v>
+      </c>
+      <c r="G2662" s="2">
+        <v>867.88</v>
+      </c>
+      <c r="H2662" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2662" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2662" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="K2662" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2663" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2663" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2663" s="2">
+        <v>163.71</v>
+      </c>
+      <c r="G2663" s="2">
+        <v>1029.75</v>
+      </c>
+      <c r="H2663" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2663" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2663" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2663" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2664" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2664" s="23">
+        <v>45945</v>
+      </c>
+      <c r="F2664" s="2">
+        <v>199.06</v>
+      </c>
+      <c r="G2664" s="2">
+        <v>1244.03</v>
+      </c>
+      <c r="H2664" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2664" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2664" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K2664" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2665" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2665" s="23">
+        <v>45947</v>
+      </c>
+      <c r="F2665" s="2">
+        <v>114.09099999999999</v>
+      </c>
+      <c r="G2665" s="2">
+        <v>670.85</v>
+      </c>
+      <c r="H2665" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2665" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2665" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2665" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2666" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2666" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2666" s="2">
+        <v>175.32</v>
+      </c>
+      <c r="G2666" s="2">
+        <v>1127.28</v>
+      </c>
+      <c r="H2666" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2666" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2666" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2666" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2667" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2667" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2667" s="2">
+        <v>82.78</v>
+      </c>
+      <c r="G2667" s="2">
+        <v>500</v>
+      </c>
+      <c r="H2667" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2667" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2667" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K2667" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2668" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2668" s="23">
+        <v>45946</v>
+      </c>
+      <c r="F2668" s="2">
+        <v>169.85</v>
+      </c>
+      <c r="G2668" s="2">
+        <v>983.43</v>
+      </c>
+      <c r="H2668" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2668" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2668" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K2668" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2669" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2669" s="23">
+        <v>45916</v>
+      </c>
+      <c r="F2669" s="2">
+        <v>141.97</v>
+      </c>
+      <c r="G2669" s="2">
+        <v>864.6</v>
+      </c>
+      <c r="H2669" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2669" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2669" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2669" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2670" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2670" s="23">
+        <v>45922</v>
+      </c>
+      <c r="F2670" s="2">
+        <v>114.96</v>
+      </c>
+      <c r="G2670" s="2">
+        <v>700.11</v>
+      </c>
+      <c r="H2670" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2670" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2670" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K2670" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="L2670" s="28"/>
     </row>
-    <row r="2673" spans="12:12" x14ac:dyDescent="0.25">
-      <c r="L2673" s="28" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="2674" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="2671" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2671" s="23">
+        <v>45926</v>
+      </c>
+      <c r="F2671" s="2">
+        <v>168.63</v>
+      </c>
+      <c r="G2671" s="2">
+        <v>1145</v>
+      </c>
+      <c r="H2671" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2671" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2671" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="K2671" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2672" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2672" s="23">
+        <v>45944</v>
+      </c>
+      <c r="F2672" s="2">
+        <v>160.96199999999999</v>
+      </c>
+      <c r="G2672" s="2">
+        <v>936.8</v>
+      </c>
+      <c r="H2672" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2672" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2672" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2672" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2673" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2673" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2673" s="2">
+        <v>49.68</v>
+      </c>
+      <c r="G2673" s="2">
+        <v>297.61</v>
+      </c>
+      <c r="H2673" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2673" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2673" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2673" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2673" s="28"/>
+    </row>
+    <row r="2674" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2674" s="23">
+        <v>45929</v>
+      </c>
+      <c r="F2674" s="2">
+        <v>135.947</v>
+      </c>
+      <c r="G2674" s="2">
+        <v>814.32</v>
+      </c>
+      <c r="H2674" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2674" s="12">
+        <v>45901</v>
+      </c>
+      <c r="J2674" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2674" s="2" t="s">
+        <v>111</v>
+      </c>
       <c r="L2674" s="28"/>
     </row>
-    <row r="2675" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="2675" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2675" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2675" s="2">
+        <v>143.85499999999999</v>
+      </c>
+      <c r="G2675" s="2">
+        <v>845.87</v>
+      </c>
+      <c r="H2675" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2675" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2675" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2675" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="L2675" s="28"/>
     </row>
-    <row r="2676" spans="12:12" x14ac:dyDescent="0.25">
+    <row r="2676" spans="2:12" x14ac:dyDescent="0.25">
       <c r="L2676" s="28"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-22  9:45
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1169" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11AD6616-EAAF-49F5-B597-951874DF896B}"/>
+  <xr:revisionPtr revIDLastSave="1221" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{010094F3-BE04-4A58-9790-266317330345}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8298" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8319" uniqueCount="341">
   <si>
     <t>Data</t>
   </si>
@@ -1060,6 +1060,9 @@
   <si>
     <t xml:space="preserve">REDE DOM PEDRO DE POSTOS </t>
   </si>
+  <si>
+    <t>POSTO CURINGA</t>
+  </si>
 </sst>
 </file>
 
@@ -1601,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-  <dimension ref="B1:L2676"/>
+  <dimension ref="B1:L2682"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.7109375" style="2" customWidth="1"/>
@@ -87578,7 +87581,166 @@
       <c r="L2675" s="28"/>
     </row>
     <row r="2676" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2676" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2676" s="2">
+        <v>46.508000000000003</v>
+      </c>
+      <c r="G2676" s="2">
+        <v>273.45999999999998</v>
+      </c>
+      <c r="H2676" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2676" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2676" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2676" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="L2676" s="28"/>
+    </row>
+    <row r="2677" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2677" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2677" s="2">
+        <v>139.63999999999999</v>
+      </c>
+      <c r="G2677" s="2">
+        <v>878.35</v>
+      </c>
+      <c r="H2677" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2677" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2677" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2677" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2678" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2678" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2678" s="2">
+        <v>109.88200000000001</v>
+      </c>
+      <c r="G2678" s="2">
+        <v>646.1</v>
+      </c>
+      <c r="H2678" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2678" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2678" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2678" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2679" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2679" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2679" s="2">
+        <v>138.20699999999999</v>
+      </c>
+      <c r="G2679" s="2">
+        <v>798.83</v>
+      </c>
+      <c r="H2679" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2679" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2679" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="K2679" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2680" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2680" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2680" s="2">
+        <v>166.52</v>
+      </c>
+      <c r="G2680" s="2">
+        <v>1064.06</v>
+      </c>
+      <c r="H2680" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2680" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2680" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="K2680" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2681" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2681" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2681" s="2">
+        <v>161.041</v>
+      </c>
+      <c r="G2681" s="2">
+        <v>946.92</v>
+      </c>
+      <c r="H2681" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2681" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2681" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K2681" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2682" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2682" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2682" s="2">
+        <v>186.97</v>
+      </c>
+      <c r="G2682" s="2">
+        <v>1176.0899999999999</v>
+      </c>
+      <c r="H2682" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2682" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2682" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2682" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B2:L2845" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-22 16:54
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1221" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{010094F3-BE04-4A58-9790-266317330345}"/>
+  <xr:revisionPtr revIDLastSave="1237" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95ED65FD-2498-41FB-A140-EC21A3C728FE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8319" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8325" uniqueCount="341">
   <si>
     <t>Data</t>
   </si>
@@ -1604,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-  <dimension ref="B1:L2682"/>
+  <dimension ref="B1:L2684"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.7109375" style="2" customWidth="1"/>
@@ -87742,6 +87742,52 @@
         <v>38</v>
       </c>
     </row>
+    <row r="2683" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2683" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2683" s="2">
+        <v>325.92</v>
+      </c>
+      <c r="G2683" s="2">
+        <v>2050.06</v>
+      </c>
+      <c r="H2683" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2683" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2683" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2683" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2684" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2684" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2684" s="2">
+        <v>206.45</v>
+      </c>
+      <c r="G2684" s="2">
+        <v>1298.5899999999999</v>
+      </c>
+      <c r="H2684" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2684" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2684" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2684" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:L2845" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-24 15:07
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1237" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95ED65FD-2498-41FB-A140-EC21A3C728FE}"/>
+  <xr:revisionPtr revIDLastSave="1383" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64E3E173-CF34-4C60-BC3F-F67414732361}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$B$2:$L$2845</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$B$2:$L$2849</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8325" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8382" uniqueCount="342">
   <si>
     <t>Data</t>
   </si>
@@ -1063,6 +1063,9 @@
   <si>
     <t>POSTO CURINGA</t>
   </si>
+  <si>
+    <t>POSTO NICODEMOS</t>
+  </si>
 </sst>
 </file>
 
@@ -1604,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-  <dimension ref="B1:L2684"/>
+  <dimension ref="B1:L2703"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.7109375" style="2" customWidth="1"/>
@@ -87788,8 +87791,445 @@
         <v>35</v>
       </c>
     </row>
+    <row r="2685" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2685" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2685" s="2">
+        <v>53.05</v>
+      </c>
+      <c r="G2685" s="2">
+        <v>333.7</v>
+      </c>
+      <c r="H2685" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2685" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2685" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2685" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2686" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2686" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2686" s="2">
+        <v>74.510000000000005</v>
+      </c>
+      <c r="G2686" s="2">
+        <v>483.57</v>
+      </c>
+      <c r="H2686" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2686" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2686" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2686" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2687" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2687" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2687" s="2">
+        <v>123.343</v>
+      </c>
+      <c r="G2687" s="2">
+        <v>725.25</v>
+      </c>
+      <c r="H2687" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2687" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2687" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="K2687" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="2688" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2688" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2688" s="2">
+        <v>161.69</v>
+      </c>
+      <c r="G2688" s="2">
+        <v>1101.7</v>
+      </c>
+      <c r="H2688" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2688" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2688" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2688" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2689" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2689" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2689" s="2">
+        <v>167.35</v>
+      </c>
+      <c r="G2689" s="2">
+        <v>1052.6600000000001</v>
+      </c>
+      <c r="H2689" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2689" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2689" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2689" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2690" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2690" s="23">
+        <v>45951</v>
+      </c>
+      <c r="F2690" s="2">
+        <v>152</v>
+      </c>
+      <c r="G2690" s="2">
+        <v>986.48</v>
+      </c>
+      <c r="H2690" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2690" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2690" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2690" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2691" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2691" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2691" s="2">
+        <v>85.34</v>
+      </c>
+      <c r="G2691" s="2">
+        <v>553.85</v>
+      </c>
+      <c r="H2691" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2691" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2691" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2691" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2692" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2692" s="23">
+        <v>45953</v>
+      </c>
+      <c r="F2692" s="2">
+        <v>181.48</v>
+      </c>
+      <c r="G2692" s="2">
+        <v>1177.81</v>
+      </c>
+      <c r="H2692" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2692" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2692" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2692" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2693" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2693" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2693" s="2">
+        <v>96.855000000000004</v>
+      </c>
+      <c r="G2693" s="2">
+        <v>569.51</v>
+      </c>
+      <c r="H2693" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2693" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2693" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="K2693" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2694" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2694" s="23">
+        <v>45944</v>
+      </c>
+      <c r="F2694" s="2">
+        <v>164.39</v>
+      </c>
+      <c r="G2694" s="2">
+        <v>1066.8900000000001</v>
+      </c>
+      <c r="H2694" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2694" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2694" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2694" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2695" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2695" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2695" s="2">
+        <v>218.76</v>
+      </c>
+      <c r="G2695" s="2">
+        <v>1367.26</v>
+      </c>
+      <c r="H2695" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2695" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2695" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K2695" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2696" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2696" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2696" s="2">
+        <v>158.16399999999999</v>
+      </c>
+      <c r="G2696" s="2">
+        <v>994.85</v>
+      </c>
+      <c r="H2696" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2696" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2696" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2696" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2697" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2697" s="23">
+        <v>45953</v>
+      </c>
+      <c r="F2697" s="2">
+        <v>23.87</v>
+      </c>
+      <c r="G2697" s="2">
+        <v>150.18</v>
+      </c>
+      <c r="H2697" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2697" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2697" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2697" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2698" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2698" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2698" s="2">
+        <v>124.42</v>
+      </c>
+      <c r="G2698" s="2">
+        <v>795.04</v>
+      </c>
+      <c r="H2698" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2698" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2698" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="K2698" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2699" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2699" s="23">
+        <v>45950</v>
+      </c>
+      <c r="F2699" s="2">
+        <v>188.376</v>
+      </c>
+      <c r="G2699" s="2">
+        <v>1298.5899999999999</v>
+      </c>
+      <c r="H2699" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2699" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2699" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2699" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2700" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2700" s="23">
+        <v>45952</v>
+      </c>
+      <c r="F2700" s="2">
+        <v>156.523</v>
+      </c>
+      <c r="G2700" s="2">
+        <v>920.35</v>
+      </c>
+      <c r="H2700" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2700" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2700" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="K2700" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2701" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2701" s="23">
+        <v>45953</v>
+      </c>
+      <c r="F2701" s="2">
+        <v>64.227999999999994</v>
+      </c>
+      <c r="G2701" s="2">
+        <v>377.65</v>
+      </c>
+      <c r="H2701" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2701" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2701" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="K2701" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2702" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2702" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2702" s="2">
+        <v>398.97</v>
+      </c>
+      <c r="G2702" s="2">
+        <v>2509.58</v>
+      </c>
+      <c r="H2702" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2702" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2702" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2702" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2703" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2703" s="23">
+        <v>45954</v>
+      </c>
+      <c r="F2703" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="G2703" s="2">
+        <v>89.01</v>
+      </c>
+      <c r="H2703" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2703" s="12">
+        <v>45931</v>
+      </c>
+      <c r="J2703" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2703" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B2:L2845" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
+  <autoFilter ref="B2:L2849" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-04 11:06
</commit_message>
<xml_diff>
--- a/data/combustivel.xlsx
+++ b/data/combustivel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1383" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64E3E173-CF34-4C60-BC3F-F67414732361}"/>
+  <xr:revisionPtr revIDLastSave="1387" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{324BDC0D-7ED1-48C8-BE60-A0517B0A5DE9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -1607,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}">
-  <dimension ref="B1:L2703"/>
+  <dimension ref="B1:L2704"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.7109375" style="2" customWidth="1"/>
@@ -88228,6 +88228,9 @@
         <v>25</v>
       </c>
     </row>
+    <row r="2704" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2704" s="23"/>
+    </row>
   </sheetData>
   <autoFilter ref="B2:L2849" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>